<commit_message>
Update consultant roster and resources
</commit_message>
<xml_diff>
--- a/assets/Strategy & Operations Service Lines.xlsx
+++ b/assets/Strategy & Operations Service Lines.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://impactadvisors3-my.sharepoint.com/personal/john_decicco_impact-advisors_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3887570-5F9F-46AB-8963-0B83357EFDDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B04B77D1-8DD2-4D21-86B9-73036EE244C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{AAB7EEAF-11CB-4475-B2F2-A15F99F765BD}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="483">
   <si>
     <t>Name</t>
   </si>
@@ -277,210 +277,201 @@
     <t>connie.mcneely@impact-advisors.com</t>
   </si>
   <si>
-    <t>Stephanie Zhou</t>
+    <t xml:space="preserve">Melissa Lingle </t>
+  </si>
+  <si>
+    <t>Melissa Lingle | LinkedIn</t>
+  </si>
+  <si>
+    <t>melissa.lingle@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Fernando Rubio-Mijangos</t>
+  </si>
+  <si>
+    <t>Fernando Rubio Mijangos | LinkedIn</t>
+  </si>
+  <si>
+    <t>fernando.rubiomijangos@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Jim Akimchuk</t>
+  </si>
+  <si>
+    <t>Operational Excellence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New Hampshire </t>
+  </si>
+  <si>
+    <t>James Akimchuk | LinkedIn</t>
+  </si>
+  <si>
+    <t>jim.akimchuk@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Kris Rickhoff</t>
+  </si>
+  <si>
+    <t>Illinois</t>
+  </si>
+  <si>
+    <t>Kris Rickhoff, MBA, RHIT, CDIP, CCS-P, CHRI, CRCR | LinkedIn</t>
+  </si>
+  <si>
+    <t>kristina.rickhoff@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Brian Junghans (VP)</t>
+  </si>
+  <si>
+    <t>Brian Junghans | LinkedIn</t>
+  </si>
+  <si>
+    <t>brian.junghans@impact-advisors.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elizabeth Anderson </t>
+  </si>
+  <si>
+    <t>Liz Anderson | LinkedIn</t>
+  </si>
+  <si>
+    <t>liz.anderson@impact-advisors.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Robin Bruce </t>
+  </si>
+  <si>
+    <t>Robin Bruce | LinkedIn</t>
+  </si>
+  <si>
+    <t>robin.bruce@impact-advisors.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kristin Berlin </t>
+  </si>
+  <si>
+    <t>Kristin Berlin, BSN, CRCR | LinkedIn</t>
+  </si>
+  <si>
+    <t>kristin.berlin@impact-advisors.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nicholas Lankford </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Washington </t>
+  </si>
+  <si>
+    <t>Nick Lankford | LinkedIn</t>
+  </si>
+  <si>
+    <t>nick.lankford@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Joel Hammer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ohio </t>
+  </si>
+  <si>
+    <t>Joel Hammer | LinkedIn</t>
+  </si>
+  <si>
+    <t>joel.hammer@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Kelsey Turasky</t>
+  </si>
+  <si>
+    <t>Kelsey Edmonds Turasky, MBA | LinkedIn</t>
+  </si>
+  <si>
+    <t>kelsey.turasky@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Kristen Camara</t>
+  </si>
+  <si>
+    <t xml:space="preserve">California </t>
+  </si>
+  <si>
+    <t>Kristen Camara | LinkedIn</t>
+  </si>
+  <si>
+    <t>kristen.camara@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Emily Vlietstra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Dakota </t>
+  </si>
+  <si>
+    <t>Emily Vlietstra | LinkedIn</t>
+  </si>
+  <si>
+    <t>emily.vlietstra@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Michael Sanders</t>
+  </si>
+  <si>
+    <t>Texas</t>
+  </si>
+  <si>
+    <t>Michael Sanders, MBA | LinkedIn</t>
+  </si>
+  <si>
+    <t>mike.sanders@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Andrew Kraemer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Carolina </t>
+  </si>
+  <si>
+    <t>Andrew K. | LinkedIn</t>
+  </si>
+  <si>
+    <t>andrew.kraemer@impact-advisors.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lisa Thompson </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nebraska </t>
+  </si>
+  <si>
+    <t>lisa.thompson@impact-advisors.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mindi Bolssen </t>
+  </si>
+  <si>
+    <t>Mindi B. | LinkedIn</t>
+  </si>
+  <si>
+    <t>mindi.bolssen@impact-advisors.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Christopher Owens </t>
+  </si>
+  <si>
+    <t>Chris Owens | LinkedIn</t>
+  </si>
+  <si>
+    <t>chris.owens@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Patricia Schlemmer</t>
   </si>
   <si>
     <t>New York</t>
   </si>
   <si>
-    <t>Stephanie Zhou | LinkedIn</t>
-  </si>
-  <si>
-    <t>stephanie.zhou@impact-advisors.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Melissa Lingle </t>
-  </si>
-  <si>
-    <t>Melissa Lingle | LinkedIn</t>
-  </si>
-  <si>
-    <t>melissa.lingle@impact-advisors.com</t>
-  </si>
-  <si>
-    <t>Fernando Rubio-Mijangos</t>
-  </si>
-  <si>
-    <t>Fernando Rubio Mijangos | LinkedIn</t>
-  </si>
-  <si>
-    <t>fernando.rubiomijangos@impact-advisors.com</t>
-  </si>
-  <si>
-    <t>Jim Akimchuk</t>
-  </si>
-  <si>
-    <t>Operational Excellence</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New Hampshire </t>
-  </si>
-  <si>
-    <t>James Akimchuk | LinkedIn</t>
-  </si>
-  <si>
-    <t>jim.akimchuk@impact-advisors.com</t>
-  </si>
-  <si>
-    <t>Kris Rickhoff</t>
-  </si>
-  <si>
-    <t>Illinois</t>
-  </si>
-  <si>
-    <t>Kris Rickhoff, MBA, RHIT, CDIP, CCS-P, CHRI, CRCR | LinkedIn</t>
-  </si>
-  <si>
-    <t>kristina.rickhoff@impact-advisors.com</t>
-  </si>
-  <si>
-    <t>Brian Junghans (VP)</t>
-  </si>
-  <si>
-    <t>Brian Junghans | LinkedIn</t>
-  </si>
-  <si>
-    <t>brian.junghans@impact-advisors.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elizabeth Anderson </t>
-  </si>
-  <si>
-    <t>Liz Anderson | LinkedIn</t>
-  </si>
-  <si>
-    <t>liz.anderson@impact-advisors.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Robin Bruce </t>
-  </si>
-  <si>
-    <t>Robin Bruce | LinkedIn</t>
-  </si>
-  <si>
-    <t>robin.bruce@impact-advisors.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kristin Berlin </t>
-  </si>
-  <si>
-    <t>Kristin Berlin, BSN, CRCR | LinkedIn</t>
-  </si>
-  <si>
-    <t>kristin.berlin@impact-advisors.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nicholas Lankford </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Washington </t>
-  </si>
-  <si>
-    <t>Nick Lankford | LinkedIn</t>
-  </si>
-  <si>
-    <t>nick.lankford@impact-advisors.com</t>
-  </si>
-  <si>
-    <t>Joel Hammer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ohio </t>
-  </si>
-  <si>
-    <t>Joel Hammer | LinkedIn</t>
-  </si>
-  <si>
-    <t>joel.hammer@impact-advisors.com</t>
-  </si>
-  <si>
-    <t>Kelsey Turasky</t>
-  </si>
-  <si>
-    <t>Kelsey Edmonds Turasky, MBA | LinkedIn</t>
-  </si>
-  <si>
-    <t>kelsey.turasky@impact-advisors.com</t>
-  </si>
-  <si>
-    <t>Kristen Camara</t>
-  </si>
-  <si>
-    <t xml:space="preserve">California </t>
-  </si>
-  <si>
-    <t>Kristen Camara | LinkedIn</t>
-  </si>
-  <si>
-    <t>kristen.camara@impact-advisors.com</t>
-  </si>
-  <si>
-    <t>Emily Vlietstra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">South Dakota </t>
-  </si>
-  <si>
-    <t>Emily Vlietstra | LinkedIn</t>
-  </si>
-  <si>
-    <t>emily.vlietstra@impact-advisors.com</t>
-  </si>
-  <si>
-    <t>Michael Sanders</t>
-  </si>
-  <si>
-    <t>Texas</t>
-  </si>
-  <si>
-    <t>Michael Sanders, MBA | LinkedIn</t>
-  </si>
-  <si>
-    <t>mike.sanders@impact-advisors.com</t>
-  </si>
-  <si>
-    <t>Andrew Kraemer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">South Carolina </t>
-  </si>
-  <si>
-    <t>Andrew K. | LinkedIn</t>
-  </si>
-  <si>
-    <t>andrew.kraemer@impact-advisors.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lisa Thompson </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nebraska </t>
-  </si>
-  <si>
-    <t>lisa.thompson@impact-advisors.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mindi Bolssen </t>
-  </si>
-  <si>
-    <t>Mindi B. | LinkedIn</t>
-  </si>
-  <si>
-    <t>mindi.bolssen@impact-advisors.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Christopher Owens </t>
-  </si>
-  <si>
-    <t>Chris Owens | LinkedIn</t>
-  </si>
-  <si>
-    <t>chris.owens@impact-advisors.com</t>
-  </si>
-  <si>
-    <t>Patricia Schlemmer</t>
-  </si>
-  <si>
     <t>Tricia Dockree | LinkedIn</t>
   </si>
   <si>
@@ -1351,6 +1342,9 @@
     <t xml:space="preserve">Kentucky </t>
   </si>
   <si>
+    <t>Andrea Feldmann | LinkedIn</t>
+  </si>
+  <si>
     <t>andrea.feldmann@impact-advisors.com</t>
   </si>
   <si>
@@ -1370,6 +1364,72 @@
   </si>
   <si>
     <t>jenifer.vaught@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Logan Hiskes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consultant </t>
+  </si>
+  <si>
+    <t>Logan Hiskes | LinkedIn</t>
+  </si>
+  <si>
+    <t>logan.hiskes@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Martin You</t>
+  </si>
+  <si>
+    <t>Martin You | LinkedIn</t>
+  </si>
+  <si>
+    <t>martin.you@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Akshita Ponnuru</t>
+  </si>
+  <si>
+    <t>Akshita Ponnuru | LinkedIn</t>
+  </si>
+  <si>
+    <t>akshita.ponnuru@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Hayden Keller</t>
+  </si>
+  <si>
+    <t>Hayden Keller, CRCR | LinkedIn</t>
+  </si>
+  <si>
+    <t>hayden.keller@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Lily Notes</t>
+  </si>
+  <si>
+    <t>Lily Notes | LinkedIn</t>
+  </si>
+  <si>
+    <t>lily.notes@impact-advisors.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khushi Patel </t>
+  </si>
+  <si>
+    <t>Khushi Patel, CRCR | LinkedIn</t>
+  </si>
+  <si>
+    <t>khushi.patel@impact-advisors.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sanya Patel </t>
+  </si>
+  <si>
+    <t>Sanya Patel | LinkedIn</t>
+  </si>
+  <si>
+    <t>sanya.patel@impact-advisors.com</t>
   </si>
   <si>
     <r>
@@ -1530,18 +1590,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1569,19 +1623,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1601,8 +1654,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}" name="Table1" displayName="Table1" ref="A1:F133" totalsRowShown="0">
-  <autoFilter ref="A1:F133" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}" name="Table1" displayName="Table1" ref="A1:F138" totalsRowShown="0">
+  <autoFilter ref="A1:F138" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{B7225A69-4070-43CE-AFA1-930CE8ABA093}" name="Name"/>
     <tableColumn id="2" xr3:uid="{74BF9A37-C28E-424C-A808-B2BBA42CFA48}" name="Service Line"/>
@@ -1981,7 +2034,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09DBBB96-A9E5-4CC1-B781-70890184EE77}">
-  <dimension ref="A1:I133"/>
+  <dimension ref="A1:I138"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -1990,6 +2043,7 @@
     <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="55.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="40.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="48.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -2388,71 +2442,71 @@
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="3" t="s">
+      <c r="A20" t="s">
         <v>78</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B20" t="s">
         <v>57</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" t="s">
+        <v>71</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="F20" t="s">
         <v>80</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B21" t="s">
         <v>57</v>
       </c>
       <c r="C21" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D21" t="s">
-        <v>71</v>
-      </c>
-      <c r="E21" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="F21" t="s">
         <v>83</v>
       </c>
-      <c r="F21" t="s">
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" s="3" t="s">
+      <c r="B22" t="s">
         <v>85</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E22" s="4" t="s">
+      <c r="C22" t="s">
+        <v>8</v>
+      </c>
+      <c r="D22" t="s">
         <v>86</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="E22" s="1" t="s">
         <v>87</v>
+      </c>
+      <c r="F22" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B23" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C23" t="s">
         <v>8</v>
@@ -2472,93 +2526,93 @@
         <v>93</v>
       </c>
       <c r="B24" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C24" t="s">
         <v>8</v>
       </c>
       <c r="D24" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="F24" t="s">
         <v>95</v>
-      </c>
-      <c r="F24" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
+        <v>96</v>
+      </c>
+      <c r="B25" t="s">
+        <v>85</v>
+      </c>
+      <c r="C25" t="s">
+        <v>13</v>
+      </c>
+      <c r="D25" t="s">
+        <v>53</v>
+      </c>
+      <c r="E25" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="B25" t="s">
-        <v>89</v>
-      </c>
-      <c r="C25" t="s">
-        <v>8</v>
-      </c>
-      <c r="D25" t="s">
-        <v>38</v>
-      </c>
-      <c r="E25" s="1" t="s">
+      <c r="F25" t="s">
         <v>98</v>
-      </c>
-      <c r="F25" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B26" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C26" t="s">
         <v>13</v>
       </c>
       <c r="D26" t="s">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E26" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="F26" t="s">
         <v>101</v>
-      </c>
-      <c r="F26" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B27" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C27" t="s">
         <v>13</v>
       </c>
       <c r="D27" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E27" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F27" t="s">
         <v>104</v>
-      </c>
-      <c r="F27" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B28" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C28" t="s">
         <v>13</v>
       </c>
       <c r="D28" t="s">
-        <v>53</v>
+        <v>106</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>107</v>
@@ -2572,7 +2626,7 @@
         <v>109</v>
       </c>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C29" t="s">
         <v>13</v>
@@ -2592,33 +2646,33 @@
         <v>113</v>
       </c>
       <c r="B30" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C30" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D30" t="s">
+        <v>90</v>
+      </c>
+      <c r="E30" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="F30" t="s">
         <v>115</v>
-      </c>
-      <c r="F30" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B31" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C31" t="s">
         <v>17</v>
       </c>
       <c r="D31" t="s">
-        <v>94</v>
+        <v>117</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>118</v>
@@ -2632,7 +2686,7 @@
         <v>120</v>
       </c>
       <c r="B32" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C32" t="s">
         <v>17</v>
@@ -2652,7 +2706,7 @@
         <v>124</v>
       </c>
       <c r="B33" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C33" t="s">
         <v>17</v>
@@ -2672,7 +2726,7 @@
         <v>128</v>
       </c>
       <c r="B34" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C34" t="s">
         <v>17</v>
@@ -2692,7 +2746,7 @@
         <v>132</v>
       </c>
       <c r="B35" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C35" t="s">
         <v>17</v>
@@ -2700,63 +2754,63 @@
       <c r="D35" t="s">
         <v>133</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="E35" s="3"/>
+      <c r="F35" t="s">
         <v>134</v>
-      </c>
-      <c r="F35" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B36" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C36" t="s">
         <v>17</v>
       </c>
       <c r="D36" t="s">
+        <v>49</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F36" t="s">
         <v>137</v>
-      </c>
-      <c r="E36" s="5"/>
-      <c r="F36" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B37" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C37" t="s">
         <v>17</v>
       </c>
       <c r="D37" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F37" t="s">
         <v>140</v>
-      </c>
-      <c r="F37" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B38" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C38" t="s">
         <v>17</v>
       </c>
       <c r="D38" t="s">
-        <v>27</v>
+        <v>142</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>143</v>
@@ -2770,53 +2824,53 @@
         <v>145</v>
       </c>
       <c r="B39" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C39" t="s">
         <v>17</v>
       </c>
       <c r="D39" t="s">
-        <v>79</v>
+        <v>146</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F39" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B40" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C40" t="s">
         <v>17</v>
       </c>
       <c r="D40" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F40" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B41" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C41" t="s">
         <v>17</v>
       </c>
       <c r="D41" t="s">
-        <v>153</v>
+        <v>49</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>154</v>
@@ -2830,13 +2884,13 @@
         <v>156</v>
       </c>
       <c r="B42" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C42" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D42" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>157</v>
@@ -2850,13 +2904,13 @@
         <v>159</v>
       </c>
       <c r="B43" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C43" t="s">
         <v>22</v>
       </c>
       <c r="D43" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>160</v>
@@ -2870,73 +2924,73 @@
         <v>162</v>
       </c>
       <c r="B44" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C44" t="s">
         <v>22</v>
       </c>
       <c r="D44" t="s">
-        <v>53</v>
+        <v>163</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F44" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="45" spans="1:6">
       <c r="A45" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B45" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C45" t="s">
         <v>22</v>
       </c>
       <c r="D45" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F45" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="46" spans="1:6">
       <c r="A46" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B46" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C46" t="s">
         <v>22</v>
       </c>
       <c r="D46" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F46" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="47" spans="1:6">
       <c r="A47" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B47" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C47" t="s">
         <v>22</v>
       </c>
       <c r="D47" t="s">
-        <v>174</v>
+        <v>53</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>175</v>
@@ -2950,13 +3004,13 @@
         <v>177</v>
       </c>
       <c r="B48" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C48" t="s">
         <v>22</v>
       </c>
       <c r="D48" t="s">
-        <v>53</v>
+        <v>125</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>178</v>
@@ -2970,33 +3024,33 @@
         <v>180</v>
       </c>
       <c r="B49" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C49" t="s">
         <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>129</v>
+        <v>181</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F49" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="50" spans="1:6">
       <c r="A50" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B50" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C50" t="s">
         <v>22</v>
       </c>
       <c r="D50" t="s">
-        <v>184</v>
+        <v>171</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>185</v>
@@ -3010,13 +3064,13 @@
         <v>187</v>
       </c>
       <c r="B51" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C51" t="s">
         <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>174</v>
+        <v>71</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>188</v>
@@ -3030,33 +3084,33 @@
         <v>190</v>
       </c>
       <c r="B52" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C52" t="s">
         <v>22</v>
       </c>
       <c r="D52" t="s">
-        <v>71</v>
+        <v>191</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F52" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="53" spans="1:6">
       <c r="A53" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B53" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C53" t="s">
         <v>22</v>
       </c>
       <c r="D53" t="s">
-        <v>194</v>
+        <v>71</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>195</v>
@@ -3070,13 +3124,13 @@
         <v>197</v>
       </c>
       <c r="B54" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C54" t="s">
         <v>22</v>
       </c>
       <c r="D54" t="s">
-        <v>71</v>
+        <v>9</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>198</v>
@@ -3090,13 +3144,13 @@
         <v>200</v>
       </c>
       <c r="B55" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C55" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D55" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>201</v>
@@ -3110,13 +3164,13 @@
         <v>203</v>
       </c>
       <c r="B56" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C56" t="s">
         <v>45</v>
       </c>
       <c r="D56" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>204</v>
@@ -3130,79 +3184,79 @@
         <v>206</v>
       </c>
       <c r="B57" t="s">
-        <v>89</v>
+        <v>207</v>
       </c>
       <c r="C57" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="D57" t="s">
-        <v>53</v>
+        <v>9</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="F57" t="s">
         <v>208</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B58" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C58" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D58" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="F58" s="1" t="s">
+      <c r="F58" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="59" spans="1:6">
-      <c r="A59" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="C59" s="3" t="s">
+      <c r="A59" t="s">
+        <v>213</v>
+      </c>
+      <c r="B59" t="s">
+        <v>207</v>
+      </c>
+      <c r="C59" t="s">
         <v>22</v>
       </c>
-      <c r="D59" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="E59" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="F59" s="3" t="s">
-        <v>81</v>
+      <c r="D59" t="s">
+        <v>9</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="F59" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="60" spans="1:6">
       <c r="A60" t="s">
-        <v>213</v>
+        <v>81</v>
       </c>
       <c r="B60" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C60" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D60" t="s">
-        <v>38</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>214</v>
+        <v>9</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>82</v>
       </c>
       <c r="F60" t="s">
-        <v>215</v>
+        <v>83</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -3210,259 +3264,259 @@
         <v>216</v>
       </c>
       <c r="B61" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="C61" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D61" t="s">
-        <v>9</v>
+        <v>117</v>
       </c>
       <c r="E61" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F61" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6">
+      <c r="A62" t="s">
+        <v>220</v>
+      </c>
+      <c r="B62" t="s">
         <v>217</v>
       </c>
-      <c r="F61" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6">
-      <c r="A62" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B62" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="C62" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D62" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E62" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F62" s="3" t="s">
-        <v>87</v>
+      <c r="C62" t="s">
+        <v>8</v>
+      </c>
+      <c r="D62" t="s">
+        <v>71</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B63" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C63" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D63" t="s">
-        <v>121</v>
+        <v>90</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F63" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="64" spans="1:6">
       <c r="A64" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B64" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C64" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D64" t="s">
-        <v>71</v>
+        <v>227</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>225</v>
+        <v>228</v>
+      </c>
+      <c r="F64" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="65" spans="1:6">
       <c r="A65" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="B65" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C65" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D65" t="s">
-        <v>94</v>
+        <v>142</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="F65" t="s">
-        <v>228</v>
+        <v>231</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="66" spans="1:6">
       <c r="A66" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="B66" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C66" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="D66" t="s">
-        <v>230</v>
+        <v>90</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="F66" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="67" spans="1:6">
       <c r="A67" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B67" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C67" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D67" t="s">
-        <v>79</v>
+        <v>167</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="68" spans="1:6">
       <c r="A68" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B68" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C68" t="s">
         <v>45</v>
       </c>
       <c r="D68" t="s">
-        <v>94</v>
+        <v>163</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="F68" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="69" spans="1:6">
       <c r="A69" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B69" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C69" t="s">
         <v>45</v>
       </c>
       <c r="D69" t="s">
-        <v>170</v>
+        <v>243</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="F69" s="1" t="s">
-        <v>241</v>
+        <v>244</v>
+      </c>
+      <c r="F69" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="70" spans="1:6">
       <c r="A70" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B70" t="s">
-        <v>220</v>
+        <v>247</v>
       </c>
       <c r="C70" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="D70" t="s">
-        <v>166</v>
+        <v>27</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="F70" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
     </row>
     <row r="71" spans="1:6">
       <c r="A71" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="B71" t="s">
-        <v>220</v>
+        <v>247</v>
       </c>
       <c r="C71" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="D71" t="s">
-        <v>246</v>
+        <v>150</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="F71" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
     </row>
     <row r="72" spans="1:6">
       <c r="A72" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B72" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C72" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D72" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="F72" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="73" spans="1:6">
       <c r="A73" t="s">
-        <v>253</v>
+        <v>60</v>
       </c>
       <c r="B73" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C73" t="s">
         <v>13</v>
       </c>
       <c r="D73" t="s">
-        <v>153</v>
+        <v>53</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>254</v>
+        <v>61</v>
       </c>
       <c r="F73" t="s">
-        <v>255</v>
+        <v>62</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -3470,10 +3524,10 @@
         <v>256</v>
       </c>
       <c r="B74" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C74" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D74" t="s">
         <v>9</v>
@@ -3487,82 +3541,82 @@
     </row>
     <row r="75" spans="1:6">
       <c r="A75" t="s">
-        <v>60</v>
+        <v>259</v>
       </c>
       <c r="B75" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C75" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D75" t="s">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>61</v>
+        <v>260</v>
       </c>
       <c r="F75" t="s">
-        <v>62</v>
+        <v>261</v>
       </c>
     </row>
     <row r="76" spans="1:6">
       <c r="A76" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B76" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C76" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D76" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="F76" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="77" spans="1:6">
       <c r="A77" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B77" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C77" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D77" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F77" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="78" spans="1:6">
       <c r="A78" t="s">
-        <v>265</v>
+        <v>78</v>
       </c>
       <c r="B78" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C78" t="s">
         <v>22</v>
       </c>
       <c r="D78" t="s">
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>266</v>
+        <v>79</v>
       </c>
       <c r="F78" t="s">
-        <v>267</v>
+        <v>80</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -3570,10 +3624,10 @@
         <v>268</v>
       </c>
       <c r="B79" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C79" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D79" t="s">
         <v>9</v>
@@ -3587,1078 +3641,1180 @@
     </row>
     <row r="80" spans="1:6">
       <c r="A80" t="s">
-        <v>82</v>
+        <v>271</v>
       </c>
       <c r="B80" t="s">
-        <v>250</v>
+        <v>272</v>
       </c>
       <c r="C80" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D80" t="s">
-        <v>71</v>
+        <v>273</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>83</v>
+        <v>274</v>
       </c>
       <c r="F80" t="s">
-        <v>84</v>
+        <v>275</v>
       </c>
     </row>
     <row r="81" spans="1:6">
       <c r="A81" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="B81" t="s">
-        <v>250</v>
+        <v>272</v>
       </c>
       <c r="C81" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="D81" t="s">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="F81" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
     </row>
     <row r="82" spans="1:6">
       <c r="A82" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="B82" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C82" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D82" t="s">
-        <v>276</v>
+        <v>75</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F82" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
     </row>
     <row r="83" spans="1:6">
       <c r="A83" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B83" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C83" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D83" t="s">
-        <v>49</v>
+        <v>75</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="F83" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
     <row r="84" spans="1:6">
       <c r="A84" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B84" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C84" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D84" t="s">
         <v>75</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="F84" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
     </row>
     <row r="85" spans="1:6">
       <c r="A85" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B85" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C85" t="s">
         <v>17</v>
       </c>
       <c r="D85" t="s">
-        <v>75</v>
+        <v>27</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="F85" t="s">
-        <v>287</v>
+        <v>289</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="86" spans="1:6">
       <c r="A86" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B86" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C86" t="s">
         <v>17</v>
       </c>
       <c r="D86" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="F86" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
     </row>
     <row r="87" spans="1:6">
       <c r="A87" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B87" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C87" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D87" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="F87" s="1" t="s">
-        <v>293</v>
+        <v>295</v>
+      </c>
+      <c r="F87" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="88" spans="1:6">
       <c r="A88" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B88" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C88" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D88" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F88" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
     </row>
     <row r="89" spans="1:6">
       <c r="A89" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B89" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C89" t="s">
         <v>22</v>
       </c>
       <c r="D89" t="s">
-        <v>23</v>
+        <v>125</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F89" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
     </row>
     <row r="90" spans="1:6">
       <c r="A90" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="B90" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C90" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D90" t="s">
-        <v>9</v>
+        <v>304</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="F90" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
     </row>
     <row r="91" spans="1:6">
       <c r="A91" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="B91" t="s">
-        <v>275</v>
+        <v>308</v>
       </c>
       <c r="C91" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D91" t="s">
-        <v>129</v>
+        <v>75</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="F91" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
     </row>
     <row r="92" spans="1:6">
       <c r="A92" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="B92" t="s">
-        <v>275</v>
+        <v>308</v>
       </c>
       <c r="C92" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="D92" t="s">
-        <v>307</v>
-      </c>
-      <c r="E92" s="1" t="s">
-        <v>308</v>
-      </c>
+        <v>18</v>
+      </c>
+      <c r="E92" s="3"/>
       <c r="F92" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
     </row>
     <row r="93" spans="1:6">
       <c r="A93" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B93" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C93" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D93" t="s">
-        <v>75</v>
+        <v>125</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F93" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="94" spans="1:6">
       <c r="A94" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B94" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C94" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D94" t="s">
-        <v>18</v>
-      </c>
-      <c r="E94" s="5"/>
+        <v>171</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>317</v>
+      </c>
       <c r="F94" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
     </row>
     <row r="95" spans="1:6">
       <c r="A95" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B95" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C95" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D95" t="s">
-        <v>129</v>
+        <v>320</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="F95" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
     </row>
     <row r="96" spans="1:6">
       <c r="A96" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="B96" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C96" t="s">
         <v>17</v>
       </c>
       <c r="D96" t="s">
-        <v>174</v>
+        <v>9</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="F96" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="97" spans="1:6">
       <c r="A97" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B97" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C97" t="s">
         <v>17</v>
       </c>
       <c r="D97" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="F97" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
     </row>
     <row r="98" spans="1:6">
       <c r="A98" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="B98" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C98" t="s">
         <v>17</v>
       </c>
       <c r="D98" t="s">
-        <v>9</v>
+        <v>117</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="F98" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="99" spans="1:6">
       <c r="A99" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="B99" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C99" t="s">
         <v>17</v>
       </c>
       <c r="D99" t="s">
-        <v>330</v>
+        <v>49</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F99" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
     </row>
     <row r="100" spans="1:6">
       <c r="A100" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B100" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C100" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D100" t="s">
-        <v>121</v>
+        <v>150</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="F100" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
     </row>
     <row r="101" spans="1:6">
       <c r="A101" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B101" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C101" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="D101" t="s">
-        <v>49</v>
+        <v>9</v>
       </c>
       <c r="E101" s="1" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F101" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="102" spans="1:6">
       <c r="A102" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B102" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C102" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D102" t="s">
-        <v>153</v>
+        <v>9</v>
       </c>
       <c r="E102" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="F102" t="s">
-        <v>341</v>
+        <v>343</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>344</v>
       </c>
     </row>
     <row r="103" spans="1:6">
       <c r="A103" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B103" t="s">
-        <v>311</v>
+        <v>346</v>
       </c>
       <c r="C103" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="D103" t="s">
-        <v>9</v>
+        <v>27</v>
       </c>
       <c r="E103" s="1" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="F103" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
     </row>
     <row r="104" spans="1:6">
       <c r="A104" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="B104" t="s">
-        <v>311</v>
+        <v>346</v>
       </c>
       <c r="C104" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="D104" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>346</v>
-      </c>
-      <c r="F104" s="1" t="s">
-        <v>347</v>
+        <v>350</v>
+      </c>
+      <c r="F104" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="105" spans="1:6">
       <c r="A105" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B105" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C105" t="s">
         <v>8</v>
       </c>
       <c r="D105" t="s">
-        <v>27</v>
+        <v>167</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="F105" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
     </row>
     <row r="106" spans="1:6">
       <c r="A106" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="B106" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C106" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D106" t="s">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="F106" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="107" spans="1:6">
       <c r="A107" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B107" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C107" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D107" t="s">
-        <v>170</v>
+        <v>227</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="F107" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="108" spans="1:6">
       <c r="A108" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B108" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C108" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D108" t="s">
         <v>9</v>
       </c>
       <c r="E108" s="1" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="F108" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="109" spans="1:6">
       <c r="A109" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B109" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C109" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D109" t="s">
-        <v>230</v>
+        <v>117</v>
       </c>
       <c r="E109" s="1" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="F109" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="110" spans="1:6">
       <c r="A110" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="B110" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C110" t="s">
         <v>22</v>
       </c>
       <c r="D110" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="E110" s="1" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="F110" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="111" spans="1:6">
       <c r="A111" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B111" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C111" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D111" t="s">
-        <v>121</v>
+        <v>27</v>
       </c>
       <c r="E111" s="1" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="F111" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
     </row>
     <row r="112" spans="1:6">
       <c r="A112" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="B112" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C112" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D112" t="s">
-        <v>18</v>
+        <v>129</v>
       </c>
       <c r="E112" s="1" t="s">
-        <v>371</v>
-      </c>
-      <c r="F112" t="s">
-        <v>372</v>
+        <v>374</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="113" spans="1:6">
       <c r="A113" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B113" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C113" t="s">
         <v>45</v>
       </c>
       <c r="D113" t="s">
-        <v>27</v>
+        <v>377</v>
       </c>
       <c r="E113" s="1" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="F113" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
     </row>
     <row r="114" spans="1:6">
       <c r="A114" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="B114" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C114" t="s">
         <v>45</v>
       </c>
       <c r="D114" t="s">
-        <v>133</v>
+        <v>9</v>
       </c>
       <c r="E114" s="1" t="s">
-        <v>377</v>
-      </c>
-      <c r="F114" s="1" t="s">
-        <v>378</v>
+        <v>381</v>
+      </c>
+      <c r="F114" t="s">
+        <v>382</v>
       </c>
     </row>
     <row r="115" spans="1:6">
       <c r="A115" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="B115" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C115" t="s">
         <v>45</v>
       </c>
       <c r="D115" t="s">
-        <v>380</v>
+        <v>163</v>
       </c>
       <c r="E115" s="1" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="F115" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
     </row>
     <row r="116" spans="1:6">
       <c r="A116" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="B116" t="s">
-        <v>349</v>
+        <v>387</v>
       </c>
       <c r="C116" t="s">
-        <v>45</v>
+        <v>388</v>
       </c>
       <c r="D116" t="s">
-        <v>9</v>
+        <v>320</v>
       </c>
       <c r="E116" s="1" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="F116" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
     </row>
     <row r="117" spans="1:6">
       <c r="A117" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="B117" t="s">
-        <v>349</v>
+        <v>387</v>
       </c>
       <c r="C117" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="D117" t="s">
-        <v>166</v>
+        <v>125</v>
       </c>
       <c r="E117" s="1" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="F117" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
     </row>
     <row r="118" spans="1:6">
       <c r="A118" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="B118" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C118" t="s">
-        <v>391</v>
+        <v>8</v>
       </c>
       <c r="D118" t="s">
-        <v>323</v>
+        <v>395</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="F118" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
     </row>
     <row r="119" spans="1:6">
       <c r="A119" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="B119" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C119" t="s">
-        <v>8</v>
+        <v>399</v>
       </c>
       <c r="D119" t="s">
-        <v>129</v>
+        <v>18</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="F119" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
     </row>
     <row r="120" spans="1:6">
       <c r="A120" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="B120" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C120" t="s">
-        <v>8</v>
+        <v>403</v>
       </c>
       <c r="D120" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="F120" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
     </row>
     <row r="121" spans="1:6">
       <c r="A121" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="B121" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C121" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D121" t="s">
-        <v>18</v>
+        <v>395</v>
       </c>
       <c r="E121" s="1" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="F121" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
     </row>
     <row r="122" spans="1:6">
       <c r="A122" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B122" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C122" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="D122" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="E122" s="1" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="F122" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
     </row>
     <row r="123" spans="1:6">
       <c r="A123" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="B123" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C123" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="D123" t="s">
-        <v>398</v>
+        <v>106</v>
       </c>
       <c r="E123" s="1" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="F123" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="124" spans="1:6">
       <c r="A124" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="B124" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C124" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="D124" t="s">
-        <v>407</v>
+        <v>49</v>
       </c>
       <c r="E124" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="F124" t="s">
-        <v>415</v>
+        <v>417</v>
+      </c>
+      <c r="F124" s="5" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="125" spans="1:6">
       <c r="A125" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="B125" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C125" t="s">
-        <v>406</v>
+        <v>13</v>
       </c>
       <c r="D125" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="E125" s="1" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="F125" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
     </row>
     <row r="126" spans="1:6">
       <c r="A126" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="B126" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C126" t="s">
-        <v>406</v>
+        <v>13</v>
       </c>
       <c r="D126" t="s">
-        <v>49</v>
+        <v>64</v>
       </c>
       <c r="E126" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="F126" s="7" t="s">
-        <v>421</v>
+        <v>423</v>
+      </c>
+      <c r="F126" t="s">
+        <v>424</v>
       </c>
     </row>
     <row r="127" spans="1:6">
       <c r="A127" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="B127" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C127" t="s">
         <v>13</v>
       </c>
       <c r="D127" t="s">
-        <v>90</v>
+        <v>167</v>
       </c>
       <c r="E127" s="1" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="F127" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
     </row>
     <row r="128" spans="1:6">
       <c r="A128" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="B128" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C128" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="D128" t="s">
-        <v>64</v>
+        <v>86</v>
       </c>
       <c r="E128" s="1" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="F128" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
     </row>
     <row r="129" spans="1:6">
       <c r="A129" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="B129" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C129" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D129" t="s">
-        <v>170</v>
+        <v>432</v>
       </c>
       <c r="E129" s="1" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="F129" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
     </row>
     <row r="130" spans="1:6">
       <c r="A130" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="B130" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C130" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="D130" t="s">
-        <v>90</v>
+        <v>167</v>
       </c>
       <c r="E130" s="1" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="F130" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
     </row>
     <row r="131" spans="1:6">
       <c r="A131" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="B131" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C131" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D131" t="s">
-        <v>435</v>
-      </c>
-      <c r="E131" s="5"/>
+        <v>273</v>
+      </c>
+      <c r="E131" s="1" t="s">
+        <v>439</v>
+      </c>
       <c r="F131" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
     </row>
     <row r="132" spans="1:6">
       <c r="A132" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="B132" t="s">
-        <v>390</v>
+        <v>308</v>
       </c>
       <c r="C132" t="s">
-        <v>22</v>
+        <v>442</v>
       </c>
       <c r="D132" t="s">
-        <v>170</v>
-      </c>
-      <c r="E132" s="1" t="s">
-        <v>438</v>
+        <v>9</v>
+      </c>
+      <c r="E132" s="6" t="s">
+        <v>443</v>
       </c>
       <c r="F132" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
     </row>
     <row r="133" spans="1:6">
       <c r="A133" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
       <c r="B133" t="s">
-        <v>390</v>
+        <v>7</v>
       </c>
       <c r="C133" t="s">
-        <v>45</v>
+        <v>442</v>
       </c>
       <c r="D133" t="s">
-        <v>276</v>
-      </c>
-      <c r="E133" s="1" t="s">
-        <v>441</v>
+        <v>9</v>
+      </c>
+      <c r="E133" s="6" t="s">
+        <v>446</v>
       </c>
       <c r="F133" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6">
+      <c r="A134" t="s">
+        <v>448</v>
+      </c>
+      <c r="B134" t="s">
+        <v>7</v>
+      </c>
+      <c r="C134" t="s">
         <v>442</v>
+      </c>
+      <c r="D134" t="s">
+        <v>9</v>
+      </c>
+      <c r="E134" s="6" t="s">
+        <v>449</v>
+      </c>
+      <c r="F134" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6">
+      <c r="A135" t="s">
+        <v>451</v>
+      </c>
+      <c r="B135" t="s">
+        <v>346</v>
+      </c>
+      <c r="C135" t="s">
+        <v>442</v>
+      </c>
+      <c r="D135" t="s">
+        <v>9</v>
+      </c>
+      <c r="E135" s="6" t="s">
+        <v>452</v>
+      </c>
+      <c r="F135" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6">
+      <c r="A136" t="s">
+        <v>454</v>
+      </c>
+      <c r="B136" t="s">
+        <v>346</v>
+      </c>
+      <c r="C136" t="s">
+        <v>442</v>
+      </c>
+      <c r="D136" t="s">
+        <v>9</v>
+      </c>
+      <c r="E136" s="6" t="s">
+        <v>455</v>
+      </c>
+      <c r="F136" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6">
+      <c r="A137" t="s">
+        <v>457</v>
+      </c>
+      <c r="B137" t="s">
+        <v>207</v>
+      </c>
+      <c r="C137" t="s">
+        <v>442</v>
+      </c>
+      <c r="D137" t="s">
+        <v>9</v>
+      </c>
+      <c r="E137" s="6" t="s">
+        <v>458</v>
+      </c>
+      <c r="F137" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6">
+      <c r="A138" t="s">
+        <v>460</v>
+      </c>
+      <c r="B138" t="s">
+        <v>7</v>
+      </c>
+      <c r="C138" t="s">
+        <v>442</v>
+      </c>
+      <c r="D138" t="s">
+        <v>9</v>
+      </c>
+      <c r="E138" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="F138" t="s">
+        <v>462</v>
       </c>
     </row>
   </sheetData>
@@ -4681,130 +4837,136 @@
     <hyperlink ref="E17" r:id="rId16" display="https://www.linkedin.com/in/alec-farmer-59805190/" xr:uid="{DFD4D7B0-1B2F-4A18-A087-2914B200A19C}"/>
     <hyperlink ref="E18" r:id="rId17" display="https://www.linkedin.com/in/michellesilverrn/" xr:uid="{DA2E1C9B-4AC6-4E1E-9135-7871A9F6FDC5}"/>
     <hyperlink ref="E19" r:id="rId18" display="https://www.linkedin.com/in/connieblackford/" xr:uid="{6A200137-9BD8-4454-BA48-494E2E208EC1}"/>
-    <hyperlink ref="E20" r:id="rId19" display="https://www.linkedin.com/in/stephaniezhou7/" xr:uid="{45137931-AE99-488B-97BF-4F367D17DFA8}"/>
-    <hyperlink ref="E21" r:id="rId20" display="https://www.linkedin.com/in/melissa-lingle-aa59b421/" xr:uid="{E86AA71B-B340-47F5-ABAB-05FEF52EA191}"/>
-    <hyperlink ref="E22" r:id="rId21" display="https://www.linkedin.com/in/fernando-rubio-mijangos-96170abb/?locale=en" xr:uid="{895406EA-0F71-461A-A610-5599446B7A3E}"/>
-    <hyperlink ref="E23" r:id="rId22" display="https://www.linkedin.com/in/james-akimchuk-8427804/" xr:uid="{57E51B5B-365E-4D29-9BAA-0509EF0C8F5D}"/>
-    <hyperlink ref="E24" r:id="rId23" display="https://www.linkedin.com/in/kris-rickhoff-mba-rhit/" xr:uid="{EF3716DE-9247-443A-950F-4E329F74B1CC}"/>
-    <hyperlink ref="E25" r:id="rId24" display="https://www.linkedin.com/in/brian-junghans-027759/" xr:uid="{FE1C2266-B7DF-494E-82C5-576AD309D867}"/>
-    <hyperlink ref="E26" r:id="rId25" display="https://www.linkedin.com/in/liz-anderson-it-project-manager/" xr:uid="{3CAC6815-B3A2-4537-BD28-7B77497F01E4}"/>
-    <hyperlink ref="E27" r:id="rId26" display="https://www.linkedin.com/in/robin-bruce-529a1a68/" xr:uid="{16746B28-9190-448F-92A6-CF89D995B1D4}"/>
-    <hyperlink ref="E28" r:id="rId27" display="https://www.linkedin.com/in/kristin-berlin-bsn-crcr-8334896/" xr:uid="{FD258DDB-6394-4AD7-A3EF-79C944FE420F}"/>
-    <hyperlink ref="E29" r:id="rId28" display="https://www.linkedin.com/in/nick-lankford-3659634/" xr:uid="{F81120C3-3AA5-47E7-BB54-B99AEEF58419}"/>
-    <hyperlink ref="E30" r:id="rId29" display="https://www.linkedin.com/in/hammerjoel/" xr:uid="{03C4726A-A638-43D2-AE24-3725DBBFCE2F}"/>
-    <hyperlink ref="E31" r:id="rId30" display="https://www.linkedin.com/in/kelseyedmonds/" xr:uid="{A1C99F42-9F9C-4DBE-8D61-86C28BDA8008}"/>
-    <hyperlink ref="E32" r:id="rId31" display="https://www.linkedin.com/in/kristen-camara/" xr:uid="{9148163F-F27A-41C4-A77D-17903E1419D1}"/>
-    <hyperlink ref="E33" r:id="rId32" display="https://www.linkedin.com/in/emily-vlietstra-984a98266/" xr:uid="{54C951ED-27F9-4D9B-BA29-998BF4BC8123}"/>
-    <hyperlink ref="E34" r:id="rId33" display="https://www.linkedin.com/in/michael-sanders-mba-29738711/" xr:uid="{B693B7AF-235E-4369-89B2-0B0C8B7C06A2}"/>
-    <hyperlink ref="E35" r:id="rId34" display="https://www.linkedin.com/in/andrew-k-53661935/" xr:uid="{0FDC3D24-98C9-4B9B-BC62-5A9A9262FEB8}"/>
-    <hyperlink ref="E37" r:id="rId35" display="https://www.linkedin.com/in/mindi-b-2a36488/" xr:uid="{07519F33-5265-4F3F-B67A-D9D2D8715172}"/>
-    <hyperlink ref="E38" r:id="rId36" display="https://www.linkedin.com/in/chris-owens-a322a3b/" xr:uid="{78434CD6-B69E-4017-8B25-7A11110B2EF1}"/>
-    <hyperlink ref="E40" r:id="rId37" display="https://www.linkedin.com/in/stuart-fedderson-mba-59953753/" xr:uid="{4682DF4A-C95A-4DA7-BEE9-541EA61C4279}"/>
-    <hyperlink ref="E41" r:id="rId38" display="https://www.linkedin.com/in/mitch-valentine-093866152/" xr:uid="{09C2F5D3-AC60-4D53-ACDF-2DED91F4D7CA}"/>
-    <hyperlink ref="E42" r:id="rId39" display="https://www.linkedin.com/in/kellycarrier/" xr:uid="{D25119FD-4814-45C2-9B84-B1C601BCF7DA}"/>
-    <hyperlink ref="E43" r:id="rId40" display="https://www.linkedin.com/in/chris-mullican-7547a71b/" xr:uid="{8654A23B-F674-4B10-81FF-26B2665F1CC1}"/>
-    <hyperlink ref="E44" r:id="rId41" display="https://www.linkedin.com/in/mary-wemhoff-7aa1165/" xr:uid="{0D41B544-3057-4FFC-BC1C-897756AA9CD4}"/>
-    <hyperlink ref="E45" r:id="rId42" display="https://www.linkedin.com/in/lorineu/" xr:uid="{E3B0E060-EE68-4E3C-BF23-C83469A3C6CC}"/>
-    <hyperlink ref="E46" r:id="rId43" display="https://www.linkedin.com/in/michael-berthiaume-05b2a619/" xr:uid="{184923EB-E350-4139-A6AB-686625BAF6ED}"/>
-    <hyperlink ref="E47" r:id="rId44" display="https://www.linkedin.com/in/casondwyer/" xr:uid="{5DDB0BE6-27FC-475F-8B23-A999C834E197}"/>
-    <hyperlink ref="E48" r:id="rId45" display="https://www.linkedin.com/in/leticiabugarin/" xr:uid="{A50742FA-51C6-464E-9372-C3EB598FB973}"/>
-    <hyperlink ref="E49" r:id="rId46" display="https://www.linkedin.com/in/christy4naturaloptions/" xr:uid="{6180F4F8-BF3C-4B79-89E1-3B8555E91E50}"/>
-    <hyperlink ref="E50" r:id="rId47" display="https://www.linkedin.com/in/alexgookins/" xr:uid="{8D3478D9-75C5-41F1-A4D9-19777E9F9224}"/>
-    <hyperlink ref="E51" r:id="rId48" display="https://www.linkedin.com/in/sarahharb/" xr:uid="{A42C71D2-0060-40B5-AD9F-A0EF691FFFAC}"/>
-    <hyperlink ref="E52" r:id="rId49" display="https://www.linkedin.com/in/karen-hopkins-2097b9126/" xr:uid="{F89286B8-F3A8-423C-B90C-0B0233DC9859}"/>
-    <hyperlink ref="E53" r:id="rId50" display="https://www.linkedin.com/in/cleanclaimconsulting/" xr:uid="{8F214AFF-B2D9-4DEA-BC74-1F675BEB26F1}"/>
-    <hyperlink ref="E54" r:id="rId51" display="https://www.linkedin.com/in/diane-powell-13b94733b/" xr:uid="{D95000CB-1BE3-435B-984B-A333B4B91AD9}"/>
-    <hyperlink ref="E55" r:id="rId52" display="https://www.linkedin.com/in/carl-czajczynski-mba-9bba513/" xr:uid="{516D0D0D-7281-46D1-A90F-35126FCE7D0A}"/>
-    <hyperlink ref="E56" r:id="rId53" display="https://www.linkedin.com/in/taylor-romano-07816b7b/" xr:uid="{F6FD2AFD-7D20-4D3D-ACA1-068C454D2BD8}"/>
-    <hyperlink ref="E57" r:id="rId54" display="https://www.linkedin.com/in/jj-manning-mba-7971359a/" xr:uid="{CACD0B23-8EEF-4C7B-89CE-296D421F3E16}"/>
-    <hyperlink ref="E58" r:id="rId55" display="https://www.linkedin.com/in/lily-oflaherty/" xr:uid="{ECEF1EC1-8758-4AF6-8862-06AF7E30AC67}"/>
-    <hyperlink ref="E60" r:id="rId56" display="https://www.linkedin.com/in/saakshi-thukral-610130163/" xr:uid="{5E8B0D7D-CB88-40CA-B0EE-BCA7B285AE43}"/>
-    <hyperlink ref="E61" r:id="rId57" display="https://www.linkedin.com/in/sarahstrom4/" xr:uid="{13FC0A3C-9267-41B1-BA5F-3FD1865FCBA3}"/>
-    <hyperlink ref="E63" r:id="rId58" display="https://www.linkedin.com/in/anwer-khan-9287623/" xr:uid="{47C79CFA-09B6-4B80-BAAD-5DE5A012A271}"/>
-    <hyperlink ref="E64" r:id="rId59" display="https://www.linkedin.com/in/ashraf-ash-shehata-415111/" xr:uid="{341263C8-DE59-42E8-B749-B4246BE8B717}"/>
-    <hyperlink ref="E65" r:id="rId60" display="https://www.linkedin.com/in/virginia-venable-b301a1/" xr:uid="{4363BDCF-F4F1-416F-AA70-078159B72F67}"/>
-    <hyperlink ref="E66" r:id="rId61" display="https://www.linkedin.com/in/susan-suarez-pesce-braun-dnp-msn-rn-ccm-206a0139/" xr:uid="{0824EB78-0712-4A12-9A83-927807A83C53}"/>
-    <hyperlink ref="E67" r:id="rId62" display="https://www.linkedin.com/in/sylvia-huq-22a808128/" xr:uid="{437C7B90-9839-484D-8DF8-2F78C20DF8B9}"/>
-    <hyperlink ref="E68" r:id="rId63" display="https://www.linkedin.com/in/katiedongoski/" xr:uid="{7404C168-E94C-4D2E-99F0-226C95417B8C}"/>
-    <hyperlink ref="E69" r:id="rId64" display="https://www.linkedin.com/in/yumimunkim/" xr:uid="{E5DF246A-2D79-4DB0-B23A-A8B7A98AD173}"/>
-    <hyperlink ref="E70" r:id="rId65" display="https://www.linkedin.com/in/kamranpanjwani/" xr:uid="{0EB82793-E457-4CAC-99A9-40FA66804CD6}"/>
-    <hyperlink ref="E71" r:id="rId66" display="https://www.linkedin.com/in/glennleininger/" xr:uid="{715050CE-E2E6-4100-9FD5-DC7C00D12E86}"/>
-    <hyperlink ref="E72" r:id="rId67" display="https://www.linkedin.com/in/david-leclercq-517a303/" xr:uid="{22759EA7-CB63-47F4-A7A3-29D51777876A}"/>
-    <hyperlink ref="E73" r:id="rId68" display="https://www.linkedin.com/in/justin-busby-future-of-healthcare/" xr:uid="{17263BD5-F08A-4503-9DF1-C9C50BBAAC01}"/>
-    <hyperlink ref="E74" r:id="rId69" display="https://www.linkedin.com/in/betsie-sassen-r-n-m-s-n-7a6129a/" xr:uid="{9B92D920-95BB-47D2-90AE-DE3B52FD5021}"/>
-    <hyperlink ref="E75" r:id="rId70" display="https://www.linkedin.com/in/kaye-reiter-msn-rn-ne-bc-97948061/" xr:uid="{E2C1DA8B-C73A-43C0-B69C-F38769F3839B}"/>
-    <hyperlink ref="E76" r:id="rId71" display="https://www.linkedin.com/in/maggie-mahowald-3916776b/" xr:uid="{4BB37C6C-0161-4AD3-86EE-08BDA1833870}"/>
-    <hyperlink ref="E77" r:id="rId72" display="https://www.linkedin.com/in/tom-frevert-20203817/" xr:uid="{614A9975-779F-47BD-BCB7-C331C61E952A}"/>
-    <hyperlink ref="E78" r:id="rId73" display="https://www.linkedin.com/in/ellen-verlen-05488335/" xr:uid="{5EF48923-B89C-49D0-9BAC-C77F9AC084B5}"/>
-    <hyperlink ref="E79" r:id="rId74" display="https://www.linkedin.com/in/grant-leclercq-a71686105/" xr:uid="{72CF59C7-94B2-489D-8B8E-839C5155E646}"/>
-    <hyperlink ref="E80" r:id="rId75" display="https://www.linkedin.com/in/melissa-lingle-aa59b421/" xr:uid="{4A280F2C-87BD-453E-9BEB-E661B64E5438}"/>
-    <hyperlink ref="E81" r:id="rId76" display="https://www.linkedin.com/in/tonyladas/" xr:uid="{405F13BB-7DF5-43BA-8E63-C86D3D7E503A}"/>
-    <hyperlink ref="E82" r:id="rId77" display="https://www.linkedin.com/in/ryan-s-44887675/" xr:uid="{667B058E-5BD9-4986-94A4-57A0F9EBB4CA}"/>
-    <hyperlink ref="E83" r:id="rId78" display="https://www.linkedin.com/in/zach-johnson-cc/" xr:uid="{D271F864-656D-4203-A9BA-2FC0E5C1D14D}"/>
-    <hyperlink ref="E84" r:id="rId79" display="https://www.linkedin.com/in/nick-stipanovich-22b0bb36/" xr:uid="{C10AF060-E10C-4FC8-B535-D66ACA4F8FAE}"/>
-    <hyperlink ref="E85" r:id="rId80" display="https://www.linkedin.com/in/evan-mcafee-122959339/" xr:uid="{6B7073C1-BA4F-4550-954C-FE174C139725}"/>
-    <hyperlink ref="E86" r:id="rId81" display="https://www.linkedin.com/in/andrea-chancellor-pmp-62b99b16/" xr:uid="{AEF65484-051E-4D74-91B5-D739602AC0E7}"/>
-    <hyperlink ref="E87" r:id="rId82" display="https://www.linkedin.com/in/quinnoglesby/" xr:uid="{D208F2FB-E8E5-43FC-91DC-A2F99F460BA3}"/>
-    <hyperlink ref="E88" r:id="rId83" display="https://www.linkedin.com/in/justingilliam/" xr:uid="{97C6F2BB-3792-4AFC-9D95-1469F0B71A70}"/>
-    <hyperlink ref="E89" r:id="rId84" display="https://www.linkedin.com/in/david-klinkhardt-2a31b9122/" xr:uid="{A4CBFA5A-7C5F-43B2-9C71-E489394D7991}"/>
-    <hyperlink ref="E90" r:id="rId85" display="https://www.linkedin.com/in/brett-reynolds167/" xr:uid="{C6A95569-DF27-47AF-B461-36129B135755}"/>
-    <hyperlink ref="E91" r:id="rId86" display="https://www.linkedin.com/in/michael-cusick-61198917/" xr:uid="{EAB3C25C-D01E-4230-9043-9C8563407538}"/>
-    <hyperlink ref="E92" r:id="rId87" display="https://www.linkedin.com/in/joshua-lake-mba-chfp-12b3b8119/" xr:uid="{B2652EDD-8F9F-4536-B4C1-06D47303BC30}"/>
-    <hyperlink ref="E93" r:id="rId88" display="https://www.linkedin.com/in/paige-ratliff-84207656/" xr:uid="{89327F44-3582-4C68-AFA0-85F44EFECF3E}"/>
-    <hyperlink ref="E95" r:id="rId89" display="https://www.linkedin.com/in/patty-marenghi-028929b7/" xr:uid="{53BA63D3-9EBA-4771-A5D8-714B905438EA}"/>
-    <hyperlink ref="E96" r:id="rId90" display="https://www.linkedin.com/in/johnarockwell/" xr:uid="{ACBC13EF-8E91-4DB9-ABD6-0B1CB0A269D8}"/>
-    <hyperlink ref="E97" r:id="rId91" display="https://www.linkedin.com/in/stephenliebowitz/" xr:uid="{782BBFC2-2AF5-4524-9BD2-AAAD355E7A0B}"/>
-    <hyperlink ref="E98" r:id="rId92" display="https://www.linkedin.com/in/lucietolan/" xr:uid="{9CC03798-F59A-4663-AD1C-628334C7EE02}"/>
-    <hyperlink ref="E99" r:id="rId93" display="https://www.linkedin.com/in/evanmorud/" xr:uid="{3CF6E493-4BEC-4CF5-AABF-DEF73E99F5FA}"/>
-    <hyperlink ref="E100" r:id="rId94" display="https://www.linkedin.com/in/jennifer-duyst-fnp-bc-fache-msn/" xr:uid="{4C9020A5-F72E-4295-A283-E23F1C6D1FB8}"/>
-    <hyperlink ref="E101" r:id="rId95" display="https://www.linkedin.com/in/shelly-welhouse-30915b50/" xr:uid="{EB50780A-EC96-492A-958F-4C7AE3F9ACC6}"/>
-    <hyperlink ref="E102" r:id="rId96" display="https://www.linkedin.com/in/sean-wydra-81b7791b9/" xr:uid="{9FBDCDAC-4C08-4930-A391-26C4FA8CCFC0}"/>
-    <hyperlink ref="E103" r:id="rId97" display="https://www.linkedin.com/in/shreyajeyakumar/" xr:uid="{FB501EE0-61FC-4D5D-B228-5F414BA74A7C}"/>
-    <hyperlink ref="E104" r:id="rId98" display="https://www.linkedin.com/in/henry-wood-68b270172/" xr:uid="{D89E190F-4DD0-4D84-BAF6-2C3A23A88432}"/>
-    <hyperlink ref="E105" r:id="rId99" display="https://www.linkedin.com/in/randynotes/" xr:uid="{888B481F-462C-43D6-9C4E-23A87228C08C}"/>
-    <hyperlink ref="E106" r:id="rId100" display="https://www.linkedin.com/in/doug-story-11356840/" xr:uid="{48503470-0A14-4A78-A0DD-12DC5D31090C}"/>
-    <hyperlink ref="E107" r:id="rId101" display="https://www.linkedin.com/in/william-ikier-a3956519/" xr:uid="{5DAEEA06-D91B-4493-8057-F6F7B83AF406}"/>
-    <hyperlink ref="E108" r:id="rId102" display="https://www.linkedin.com/in/candace-rogerson-6846864b/" xr:uid="{A3078A11-C3C2-4508-B4FB-90F1093B7FA8}"/>
-    <hyperlink ref="E109" r:id="rId103" display="https://www.linkedin.com/in/kaylalawrie/" xr:uid="{8904D271-EECE-41A7-9C19-CABF76B6E999}"/>
-    <hyperlink ref="E110" r:id="rId104" display="https://www.linkedin.com/in/kyle-boudreau-mba/" xr:uid="{67C04911-918E-4EAC-86B8-ACCF74B215FA}"/>
-    <hyperlink ref="E111" r:id="rId105" display="https://www.linkedin.com/in/monica-dupaix/" xr:uid="{2A702DE6-44BB-4123-A579-8F8561D31637}"/>
-    <hyperlink ref="E112" r:id="rId106" display="https://www.linkedin.com/in/samuel-depaz-87206753/" xr:uid="{FBB0030F-0A29-4BA7-AD1C-E5B82813ABD4}"/>
-    <hyperlink ref="E113" r:id="rId107" display="https://www.linkedin.com/in/lauren-thompson-73545a68/" xr:uid="{DAFA2A8D-4213-4A7B-8153-78BD0D407B67}"/>
-    <hyperlink ref="E114" r:id="rId108" display="https://www.linkedin.com/in/nicolelhaas/" xr:uid="{F9648206-5E74-466F-A7BC-1F28B3CC2D17}"/>
-    <hyperlink ref="E115" r:id="rId109" display="https://www.linkedin.com/in/paul-sirakowski/" xr:uid="{C3785549-561C-4DAD-8855-171276C80650}"/>
-    <hyperlink ref="E116" r:id="rId110" display="https://www.linkedin.com/in/jacksonkithcart/" xr:uid="{411D6BA1-9FC0-4E11-8D19-C41740475183}"/>
-    <hyperlink ref="E117" r:id="rId111" display="https://www.linkedin.com/in/catherinepark1/" xr:uid="{D3F4C2C6-C885-4503-AA56-28A1BA5454AD}"/>
-    <hyperlink ref="E118" r:id="rId112" display="https://www.linkedin.com/in/wes-arnett/" xr:uid="{E5CF6DAD-CD03-471D-9BD5-371DAD58E440}"/>
-    <hyperlink ref="E119" r:id="rId113" display="https://www.linkedin.com/in/christophermcdonald/" xr:uid="{526A4A42-1CFB-4950-866D-E71BDE746F55}"/>
-    <hyperlink ref="E120" r:id="rId114" display="https://www.linkedin.com/in/patrickoconnorjr/" xr:uid="{068E1C2A-4BD1-40B8-ACEA-E24A87BEB90A}"/>
-    <hyperlink ref="E122" r:id="rId115" display="https://www.linkedin.com/in/conyers-poole-5a719711/" xr:uid="{833A676B-E1CE-482D-A830-253F46C75A60}"/>
-    <hyperlink ref="E123" r:id="rId116" display="https://www.linkedin.com/in/darbi-shanker-2b5b18a/?skipRedirect=true" xr:uid="{6500C002-6EE0-42B0-9CAE-33C9EF0917D7}"/>
-    <hyperlink ref="E125" r:id="rId117" display="https://www.linkedin.com/in/amber-thomas-jd/" xr:uid="{66251144-533E-4A9E-8C91-470FF529CF69}"/>
-    <hyperlink ref="E126" r:id="rId118" display="https://www.linkedin.com/in/danivoss/" xr:uid="{031AC3E3-5ACC-47F0-A0DA-486554A301F0}"/>
-    <hyperlink ref="E127" r:id="rId119" display="https://www.linkedin.com/in/sarahellenrcm/" xr:uid="{2BFC6DD6-B985-48AE-9622-3E4D9324B31B}"/>
-    <hyperlink ref="E128" r:id="rId120" display="https://www.linkedin.com/in/-teresa-sutton/" xr:uid="{9800A925-F666-47EE-9FB6-FBE50622AC7B}"/>
-    <hyperlink ref="E129" r:id="rId121" display="https://www.linkedin.com/in/rgavrilles/" xr:uid="{DC2C4FA9-E9C2-4C88-B916-31D863FBC92F}"/>
-    <hyperlink ref="E130" r:id="rId122" display="https://www.linkedin.com/in/reoconnell/" xr:uid="{55DA8231-4CDF-4E0F-8DF9-7334C9B8DAFC}"/>
-    <hyperlink ref="E132" r:id="rId123" display="https://www.linkedin.com/in/coreyarmstrong1/" xr:uid="{15F5CFE4-5270-456A-9E9C-9EC74F31497E}"/>
-    <hyperlink ref="E133" r:id="rId124" display="https://www.linkedin.com/in/jenifer-vaught-742489274/" xr:uid="{7295AD66-A81B-40BC-9FAC-30BFC1BCEEE8}"/>
-    <hyperlink ref="E59" r:id="rId125" display="https://www.linkedin.com/in/stephaniezhou7/" xr:uid="{383E1828-DAA9-47C1-BE4F-91FCCEAED3AE}"/>
-    <hyperlink ref="E62" r:id="rId126" display="https://www.linkedin.com/in/fernando-rubio-mijangos-96170abb/?locale=en" xr:uid="{82E02949-9FAA-4917-A569-F91A6C46A7BA}"/>
-    <hyperlink ref="F3" r:id="rId127" xr:uid="{8BE6930C-AAAB-474C-9307-020BDA839FB3}"/>
-    <hyperlink ref="F5" r:id="rId128" xr:uid="{E10613DC-661A-4A5D-9F2C-AAECE390326A}"/>
-    <hyperlink ref="F58" r:id="rId129" xr:uid="{B73E8DA3-D774-457E-B5C9-6925C167B6AE}"/>
-    <hyperlink ref="F64" r:id="rId130" xr:uid="{10B36F5A-1B69-4B91-B5C6-C9A0F774442B}"/>
-    <hyperlink ref="F67" r:id="rId131" xr:uid="{CEABCAD5-D00D-4114-8985-B83270679455}"/>
-    <hyperlink ref="F69" r:id="rId132" xr:uid="{E7946A30-8A55-4A37-B155-B6EFB266D883}"/>
-    <hyperlink ref="F114" r:id="rId133" xr:uid="{868A966A-8C31-47FD-A98D-4C402066AFB7}"/>
-    <hyperlink ref="F87" r:id="rId134" xr:uid="{6AEF366C-9DF8-4824-89B0-4C71020C0079}"/>
-    <hyperlink ref="F104" r:id="rId135" xr:uid="{B8ACDDF3-8E66-4E78-A519-C81C929AFB2F}"/>
-    <hyperlink ref="E39" r:id="rId136" display="https://www.linkedin.com/in/tricia-dockree-821b453a/" xr:uid="{DA65C1A0-887B-453C-8B5E-C6B2C12E98D4}"/>
-    <hyperlink ref="E124" r:id="rId137" display="https://www.linkedin.com/in/kristin-costanzo-931498380/" xr:uid="{F57E52E8-84BA-4F35-97F6-09377464E399}"/>
-    <hyperlink ref="E121" r:id="rId138" display="https://www.linkedin.com/in/stephen-m-bernard/" xr:uid="{3AF57711-4517-4503-80B1-3A0F825046CD}"/>
+    <hyperlink ref="E20" r:id="rId19" display="https://www.linkedin.com/in/melissa-lingle-aa59b421/" xr:uid="{E86AA71B-B340-47F5-ABAB-05FEF52EA191}"/>
+    <hyperlink ref="E21" r:id="rId20" display="https://www.linkedin.com/in/fernando-rubio-mijangos-96170abb/?locale=en" xr:uid="{895406EA-0F71-461A-A610-5599446B7A3E}"/>
+    <hyperlink ref="E22" r:id="rId21" display="https://www.linkedin.com/in/james-akimchuk-8427804/" xr:uid="{57E51B5B-365E-4D29-9BAA-0509EF0C8F5D}"/>
+    <hyperlink ref="E23" r:id="rId22" display="https://www.linkedin.com/in/kris-rickhoff-mba-rhit/" xr:uid="{EF3716DE-9247-443A-950F-4E329F74B1CC}"/>
+    <hyperlink ref="E24" r:id="rId23" display="https://www.linkedin.com/in/brian-junghans-027759/" xr:uid="{FE1C2266-B7DF-494E-82C5-576AD309D867}"/>
+    <hyperlink ref="E25" r:id="rId24" display="https://www.linkedin.com/in/liz-anderson-it-project-manager/" xr:uid="{3CAC6815-B3A2-4537-BD28-7B77497F01E4}"/>
+    <hyperlink ref="E26" r:id="rId25" display="https://www.linkedin.com/in/robin-bruce-529a1a68/" xr:uid="{16746B28-9190-448F-92A6-CF89D995B1D4}"/>
+    <hyperlink ref="E27" r:id="rId26" display="https://www.linkedin.com/in/kristin-berlin-bsn-crcr-8334896/" xr:uid="{FD258DDB-6394-4AD7-A3EF-79C944FE420F}"/>
+    <hyperlink ref="E28" r:id="rId27" display="https://www.linkedin.com/in/nick-lankford-3659634/" xr:uid="{F81120C3-3AA5-47E7-BB54-B99AEEF58419}"/>
+    <hyperlink ref="E29" r:id="rId28" display="https://www.linkedin.com/in/hammerjoel/" xr:uid="{03C4726A-A638-43D2-AE24-3725DBBFCE2F}"/>
+    <hyperlink ref="E30" r:id="rId29" display="https://www.linkedin.com/in/kelseyedmonds/" xr:uid="{A1C99F42-9F9C-4DBE-8D61-86C28BDA8008}"/>
+    <hyperlink ref="E31" r:id="rId30" display="https://www.linkedin.com/in/kristen-camara/" xr:uid="{9148163F-F27A-41C4-A77D-17903E1419D1}"/>
+    <hyperlink ref="E32" r:id="rId31" display="https://www.linkedin.com/in/emily-vlietstra-984a98266/" xr:uid="{54C951ED-27F9-4D9B-BA29-998BF4BC8123}"/>
+    <hyperlink ref="E33" r:id="rId32" display="https://www.linkedin.com/in/michael-sanders-mba-29738711/" xr:uid="{B693B7AF-235E-4369-89B2-0B0C8B7C06A2}"/>
+    <hyperlink ref="E34" r:id="rId33" display="https://www.linkedin.com/in/andrew-k-53661935/" xr:uid="{0FDC3D24-98C9-4B9B-BC62-5A9A9262FEB8}"/>
+    <hyperlink ref="E36" r:id="rId34" display="https://www.linkedin.com/in/mindi-b-2a36488/" xr:uid="{07519F33-5265-4F3F-B67A-D9D2D8715172}"/>
+    <hyperlink ref="E37" r:id="rId35" display="https://www.linkedin.com/in/chris-owens-a322a3b/" xr:uid="{78434CD6-B69E-4017-8B25-7A11110B2EF1}"/>
+    <hyperlink ref="E39" r:id="rId36" display="https://www.linkedin.com/in/stuart-fedderson-mba-59953753/" xr:uid="{4682DF4A-C95A-4DA7-BEE9-541EA61C4279}"/>
+    <hyperlink ref="E40" r:id="rId37" display="https://www.linkedin.com/in/mitch-valentine-093866152/" xr:uid="{09C2F5D3-AC60-4D53-ACDF-2DED91F4D7CA}"/>
+    <hyperlink ref="E41" r:id="rId38" display="https://www.linkedin.com/in/kellycarrier/" xr:uid="{D25119FD-4814-45C2-9B84-B1C601BCF7DA}"/>
+    <hyperlink ref="E42" r:id="rId39" display="https://www.linkedin.com/in/chris-mullican-7547a71b/" xr:uid="{8654A23B-F674-4B10-81FF-26B2665F1CC1}"/>
+    <hyperlink ref="E43" r:id="rId40" display="https://www.linkedin.com/in/mary-wemhoff-7aa1165/" xr:uid="{0D41B544-3057-4FFC-BC1C-897756AA9CD4}"/>
+    <hyperlink ref="E44" r:id="rId41" display="https://www.linkedin.com/in/lorineu/" xr:uid="{E3B0E060-EE68-4E3C-BF23-C83469A3C6CC}"/>
+    <hyperlink ref="E45" r:id="rId42" display="https://www.linkedin.com/in/michael-berthiaume-05b2a619/" xr:uid="{184923EB-E350-4139-A6AB-686625BAF6ED}"/>
+    <hyperlink ref="E46" r:id="rId43" display="https://www.linkedin.com/in/casondwyer/" xr:uid="{5DDB0BE6-27FC-475F-8B23-A999C834E197}"/>
+    <hyperlink ref="E47" r:id="rId44" display="https://www.linkedin.com/in/leticiabugarin/" xr:uid="{A50742FA-51C6-464E-9372-C3EB598FB973}"/>
+    <hyperlink ref="E48" r:id="rId45" display="https://www.linkedin.com/in/christy4naturaloptions/" xr:uid="{6180F4F8-BF3C-4B79-89E1-3B8555E91E50}"/>
+    <hyperlink ref="E49" r:id="rId46" display="https://www.linkedin.com/in/alexgookins/" xr:uid="{8D3478D9-75C5-41F1-A4D9-19777E9F9224}"/>
+    <hyperlink ref="E50" r:id="rId47" display="https://www.linkedin.com/in/sarahharb/" xr:uid="{A42C71D2-0060-40B5-AD9F-A0EF691FFFAC}"/>
+    <hyperlink ref="E51" r:id="rId48" display="https://www.linkedin.com/in/karen-hopkins-2097b9126/" xr:uid="{F89286B8-F3A8-423C-B90C-0B0233DC9859}"/>
+    <hyperlink ref="E52" r:id="rId49" display="https://www.linkedin.com/in/cleanclaimconsulting/" xr:uid="{8F214AFF-B2D9-4DEA-BC74-1F675BEB26F1}"/>
+    <hyperlink ref="E53" r:id="rId50" display="https://www.linkedin.com/in/diane-powell-13b94733b/" xr:uid="{D95000CB-1BE3-435B-984B-A333B4B91AD9}"/>
+    <hyperlink ref="E54" r:id="rId51" display="https://www.linkedin.com/in/carl-czajczynski-mba-9bba513/" xr:uid="{516D0D0D-7281-46D1-A90F-35126FCE7D0A}"/>
+    <hyperlink ref="E55" r:id="rId52" display="https://www.linkedin.com/in/taylor-romano-07816b7b/" xr:uid="{F6FD2AFD-7D20-4D3D-ACA1-068C454D2BD8}"/>
+    <hyperlink ref="E56" r:id="rId53" display="https://www.linkedin.com/in/jj-manning-mba-7971359a/" xr:uid="{CACD0B23-8EEF-4C7B-89CE-296D421F3E16}"/>
+    <hyperlink ref="E57" r:id="rId54" display="https://www.linkedin.com/in/lily-oflaherty/" xr:uid="{ECEF1EC1-8758-4AF6-8862-06AF7E30AC67}"/>
+    <hyperlink ref="E58" r:id="rId55" display="https://www.linkedin.com/in/saakshi-thukral-610130163/" xr:uid="{5E8B0D7D-CB88-40CA-B0EE-BCA7B285AE43}"/>
+    <hyperlink ref="E59" r:id="rId56" display="https://www.linkedin.com/in/sarahstrom4/" xr:uid="{13FC0A3C-9267-41B1-BA5F-3FD1865FCBA3}"/>
+    <hyperlink ref="E61" r:id="rId57" display="https://www.linkedin.com/in/anwer-khan-9287623/" xr:uid="{47C79CFA-09B6-4B80-BAAD-5DE5A012A271}"/>
+    <hyperlink ref="E62" r:id="rId58" display="https://www.linkedin.com/in/ashraf-ash-shehata-415111/" xr:uid="{341263C8-DE59-42E8-B749-B4246BE8B717}"/>
+    <hyperlink ref="E63" r:id="rId59" display="https://www.linkedin.com/in/virginia-venable-b301a1/" xr:uid="{4363BDCF-F4F1-416F-AA70-078159B72F67}"/>
+    <hyperlink ref="E64" r:id="rId60" display="https://www.linkedin.com/in/susan-suarez-pesce-braun-dnp-msn-rn-ccm-206a0139/" xr:uid="{0824EB78-0712-4A12-9A83-927807A83C53}"/>
+    <hyperlink ref="E65" r:id="rId61" display="https://www.linkedin.com/in/sylvia-huq-22a808128/" xr:uid="{437C7B90-9839-484D-8DF8-2F78C20DF8B9}"/>
+    <hyperlink ref="E66" r:id="rId62" display="https://www.linkedin.com/in/katiedongoski/" xr:uid="{7404C168-E94C-4D2E-99F0-226C95417B8C}"/>
+    <hyperlink ref="E67" r:id="rId63" display="https://www.linkedin.com/in/yumimunkim/" xr:uid="{E5DF246A-2D79-4DB0-B23A-A8B7A98AD173}"/>
+    <hyperlink ref="E68" r:id="rId64" display="https://www.linkedin.com/in/kamranpanjwani/" xr:uid="{0EB82793-E457-4CAC-99A9-40FA66804CD6}"/>
+    <hyperlink ref="E69" r:id="rId65" display="https://www.linkedin.com/in/glennleininger/" xr:uid="{715050CE-E2E6-4100-9FD5-DC7C00D12E86}"/>
+    <hyperlink ref="E70" r:id="rId66" display="https://www.linkedin.com/in/david-leclercq-517a303/" xr:uid="{22759EA7-CB63-47F4-A7A3-29D51777876A}"/>
+    <hyperlink ref="E71" r:id="rId67" display="https://www.linkedin.com/in/justin-busby-future-of-healthcare/" xr:uid="{17263BD5-F08A-4503-9DF1-C9C50BBAAC01}"/>
+    <hyperlink ref="E72" r:id="rId68" display="https://www.linkedin.com/in/betsie-sassen-r-n-m-s-n-7a6129a/" xr:uid="{9B92D920-95BB-47D2-90AE-DE3B52FD5021}"/>
+    <hyperlink ref="E73" r:id="rId69" display="https://www.linkedin.com/in/kaye-reiter-msn-rn-ne-bc-97948061/" xr:uid="{E2C1DA8B-C73A-43C0-B69C-F38769F3839B}"/>
+    <hyperlink ref="E74" r:id="rId70" display="https://www.linkedin.com/in/maggie-mahowald-3916776b/" xr:uid="{4BB37C6C-0161-4AD3-86EE-08BDA1833870}"/>
+    <hyperlink ref="E75" r:id="rId71" display="https://www.linkedin.com/in/tom-frevert-20203817/" xr:uid="{614A9975-779F-47BD-BCB7-C331C61E952A}"/>
+    <hyperlink ref="E76" r:id="rId72" display="https://www.linkedin.com/in/ellen-verlen-05488335/" xr:uid="{5EF48923-B89C-49D0-9BAC-C77F9AC084B5}"/>
+    <hyperlink ref="E77" r:id="rId73" display="https://www.linkedin.com/in/grant-leclercq-a71686105/" xr:uid="{72CF59C7-94B2-489D-8B8E-839C5155E646}"/>
+    <hyperlink ref="E78" r:id="rId74" display="https://www.linkedin.com/in/melissa-lingle-aa59b421/" xr:uid="{4A280F2C-87BD-453E-9BEB-E661B64E5438}"/>
+    <hyperlink ref="E79" r:id="rId75" display="https://www.linkedin.com/in/tonyladas/" xr:uid="{405F13BB-7DF5-43BA-8E63-C86D3D7E503A}"/>
+    <hyperlink ref="E80" r:id="rId76" display="https://www.linkedin.com/in/ryan-s-44887675/" xr:uid="{667B058E-5BD9-4986-94A4-57A0F9EBB4CA}"/>
+    <hyperlink ref="E81" r:id="rId77" display="https://www.linkedin.com/in/zach-johnson-cc/" xr:uid="{D271F864-656D-4203-A9BA-2FC0E5C1D14D}"/>
+    <hyperlink ref="E82" r:id="rId78" display="https://www.linkedin.com/in/nick-stipanovich-22b0bb36/" xr:uid="{C10AF060-E10C-4FC8-B535-D66ACA4F8FAE}"/>
+    <hyperlink ref="E83" r:id="rId79" display="https://www.linkedin.com/in/evan-mcafee-122959339/" xr:uid="{6B7073C1-BA4F-4550-954C-FE174C139725}"/>
+    <hyperlink ref="E84" r:id="rId80" display="https://www.linkedin.com/in/andrea-chancellor-pmp-62b99b16/" xr:uid="{AEF65484-051E-4D74-91B5-D739602AC0E7}"/>
+    <hyperlink ref="E85" r:id="rId81" display="https://www.linkedin.com/in/quinnoglesby/" xr:uid="{D208F2FB-E8E5-43FC-91DC-A2F99F460BA3}"/>
+    <hyperlink ref="E86" r:id="rId82" display="https://www.linkedin.com/in/justingilliam/" xr:uid="{97C6F2BB-3792-4AFC-9D95-1469F0B71A70}"/>
+    <hyperlink ref="E87" r:id="rId83" display="https://www.linkedin.com/in/david-klinkhardt-2a31b9122/" xr:uid="{A4CBFA5A-7C5F-43B2-9C71-E489394D7991}"/>
+    <hyperlink ref="E88" r:id="rId84" display="https://www.linkedin.com/in/brett-reynolds167/" xr:uid="{C6A95569-DF27-47AF-B461-36129B135755}"/>
+    <hyperlink ref="E89" r:id="rId85" display="https://www.linkedin.com/in/michael-cusick-61198917/" xr:uid="{EAB3C25C-D01E-4230-9043-9C8563407538}"/>
+    <hyperlink ref="E90" r:id="rId86" display="https://www.linkedin.com/in/joshua-lake-mba-chfp-12b3b8119/" xr:uid="{B2652EDD-8F9F-4536-B4C1-06D47303BC30}"/>
+    <hyperlink ref="E91" r:id="rId87" display="https://www.linkedin.com/in/paige-ratliff-84207656/" xr:uid="{89327F44-3582-4C68-AFA0-85F44EFECF3E}"/>
+    <hyperlink ref="E93" r:id="rId88" display="https://www.linkedin.com/in/patty-marenghi-028929b7/" xr:uid="{53BA63D3-9EBA-4771-A5D8-714B905438EA}"/>
+    <hyperlink ref="E94" r:id="rId89" display="https://www.linkedin.com/in/johnarockwell/" xr:uid="{ACBC13EF-8E91-4DB9-ABD6-0B1CB0A269D8}"/>
+    <hyperlink ref="E95" r:id="rId90" display="https://www.linkedin.com/in/stephenliebowitz/" xr:uid="{782BBFC2-2AF5-4524-9BD2-AAAD355E7A0B}"/>
+    <hyperlink ref="E96" r:id="rId91" display="https://www.linkedin.com/in/lucietolan/" xr:uid="{9CC03798-F59A-4663-AD1C-628334C7EE02}"/>
+    <hyperlink ref="E97" r:id="rId92" display="https://www.linkedin.com/in/evanmorud/" xr:uid="{3CF6E493-4BEC-4CF5-AABF-DEF73E99F5FA}"/>
+    <hyperlink ref="E98" r:id="rId93" display="https://www.linkedin.com/in/jennifer-duyst-fnp-bc-fache-msn/" xr:uid="{4C9020A5-F72E-4295-A283-E23F1C6D1FB8}"/>
+    <hyperlink ref="E99" r:id="rId94" display="https://www.linkedin.com/in/shelly-welhouse-30915b50/" xr:uid="{EB50780A-EC96-492A-958F-4C7AE3F9ACC6}"/>
+    <hyperlink ref="E100" r:id="rId95" display="https://www.linkedin.com/in/sean-wydra-81b7791b9/" xr:uid="{9FBDCDAC-4C08-4930-A391-26C4FA8CCFC0}"/>
+    <hyperlink ref="E101" r:id="rId96" display="https://www.linkedin.com/in/shreyajeyakumar/" xr:uid="{FB501EE0-61FC-4D5D-B228-5F414BA74A7C}"/>
+    <hyperlink ref="E102" r:id="rId97" display="https://www.linkedin.com/in/henry-wood-68b270172/" xr:uid="{D89E190F-4DD0-4D84-BAF6-2C3A23A88432}"/>
+    <hyperlink ref="E103" r:id="rId98" display="https://www.linkedin.com/in/randynotes/" xr:uid="{888B481F-462C-43D6-9C4E-23A87228C08C}"/>
+    <hyperlink ref="E104" r:id="rId99" display="https://www.linkedin.com/in/doug-story-11356840/" xr:uid="{48503470-0A14-4A78-A0DD-12DC5D31090C}"/>
+    <hyperlink ref="E105" r:id="rId100" display="https://www.linkedin.com/in/william-ikier-a3956519/" xr:uid="{5DAEEA06-D91B-4493-8057-F6F7B83AF406}"/>
+    <hyperlink ref="E106" r:id="rId101" display="https://www.linkedin.com/in/candace-rogerson-6846864b/" xr:uid="{A3078A11-C3C2-4508-B4FB-90F1093B7FA8}"/>
+    <hyperlink ref="E107" r:id="rId102" display="https://www.linkedin.com/in/kaylalawrie/" xr:uid="{8904D271-EECE-41A7-9C19-CABF76B6E999}"/>
+    <hyperlink ref="E108" r:id="rId103" display="https://www.linkedin.com/in/kyle-boudreau-mba/" xr:uid="{67C04911-918E-4EAC-86B8-ACCF74B215FA}"/>
+    <hyperlink ref="E109" r:id="rId104" display="https://www.linkedin.com/in/monica-dupaix/" xr:uid="{2A702DE6-44BB-4123-A579-8F8561D31637}"/>
+    <hyperlink ref="E110" r:id="rId105" display="https://www.linkedin.com/in/samuel-depaz-87206753/" xr:uid="{FBB0030F-0A29-4BA7-AD1C-E5B82813ABD4}"/>
+    <hyperlink ref="E111" r:id="rId106" display="https://www.linkedin.com/in/lauren-thompson-73545a68/" xr:uid="{DAFA2A8D-4213-4A7B-8153-78BD0D407B67}"/>
+    <hyperlink ref="E112" r:id="rId107" display="https://www.linkedin.com/in/nicolelhaas/" xr:uid="{F9648206-5E74-466F-A7BC-1F28B3CC2D17}"/>
+    <hyperlink ref="E113" r:id="rId108" display="https://www.linkedin.com/in/paul-sirakowski/" xr:uid="{C3785549-561C-4DAD-8855-171276C80650}"/>
+    <hyperlink ref="E114" r:id="rId109" display="https://www.linkedin.com/in/jacksonkithcart/" xr:uid="{411D6BA1-9FC0-4E11-8D19-C41740475183}"/>
+    <hyperlink ref="E115" r:id="rId110" display="https://www.linkedin.com/in/catherinepark1/" xr:uid="{D3F4C2C6-C885-4503-AA56-28A1BA5454AD}"/>
+    <hyperlink ref="E116" r:id="rId111" display="https://www.linkedin.com/in/wes-arnett/" xr:uid="{E5CF6DAD-CD03-471D-9BD5-371DAD58E440}"/>
+    <hyperlink ref="E117" r:id="rId112" display="https://www.linkedin.com/in/christophermcdonald/" xr:uid="{526A4A42-1CFB-4950-866D-E71BDE746F55}"/>
+    <hyperlink ref="E118" r:id="rId113" display="https://www.linkedin.com/in/patrickoconnorjr/" xr:uid="{068E1C2A-4BD1-40B8-ACEA-E24A87BEB90A}"/>
+    <hyperlink ref="E120" r:id="rId114" display="https://www.linkedin.com/in/conyers-poole-5a719711/" xr:uid="{833A676B-E1CE-482D-A830-253F46C75A60}"/>
+    <hyperlink ref="E121" r:id="rId115" display="https://www.linkedin.com/in/darbi-shanker-2b5b18a/?skipRedirect=true" xr:uid="{6500C002-6EE0-42B0-9CAE-33C9EF0917D7}"/>
+    <hyperlink ref="E123" r:id="rId116" display="https://www.linkedin.com/in/amber-thomas-jd/" xr:uid="{66251144-533E-4A9E-8C91-470FF529CF69}"/>
+    <hyperlink ref="E124" r:id="rId117" display="https://www.linkedin.com/in/danivoss/" xr:uid="{031AC3E3-5ACC-47F0-A0DA-486554A301F0}"/>
+    <hyperlink ref="E125" r:id="rId118" display="https://www.linkedin.com/in/sarahellenrcm/" xr:uid="{2BFC6DD6-B985-48AE-9622-3E4D9324B31B}"/>
+    <hyperlink ref="E126" r:id="rId119" display="https://www.linkedin.com/in/-teresa-sutton/" xr:uid="{9800A925-F666-47EE-9FB6-FBE50622AC7B}"/>
+    <hyperlink ref="E127" r:id="rId120" display="https://www.linkedin.com/in/rgavrilles/" xr:uid="{DC2C4FA9-E9C2-4C88-B916-31D863FBC92F}"/>
+    <hyperlink ref="E128" r:id="rId121" display="https://www.linkedin.com/in/reoconnell/" xr:uid="{55DA8231-4CDF-4E0F-8DF9-7334C9B8DAFC}"/>
+    <hyperlink ref="E130" r:id="rId122" display="https://www.linkedin.com/in/coreyarmstrong1/" xr:uid="{15F5CFE4-5270-456A-9E9C-9EC74F31497E}"/>
+    <hyperlink ref="E131" r:id="rId123" display="https://www.linkedin.com/in/jenifer-vaught-742489274/" xr:uid="{7295AD66-A81B-40BC-9FAC-30BFC1BCEEE8}"/>
+    <hyperlink ref="E60" r:id="rId124" display="https://www.linkedin.com/in/fernando-rubio-mijangos-96170abb/?locale=en" xr:uid="{82E02949-9FAA-4917-A569-F91A6C46A7BA}"/>
+    <hyperlink ref="F3" r:id="rId125" xr:uid="{8BE6930C-AAAB-474C-9307-020BDA839FB3}"/>
+    <hyperlink ref="F5" r:id="rId126" xr:uid="{E10613DC-661A-4A5D-9F2C-AAECE390326A}"/>
+    <hyperlink ref="F57" r:id="rId127" xr:uid="{B73E8DA3-D774-457E-B5C9-6925C167B6AE}"/>
+    <hyperlink ref="F62" r:id="rId128" xr:uid="{10B36F5A-1B69-4B91-B5C6-C9A0F774442B}"/>
+    <hyperlink ref="F65" r:id="rId129" xr:uid="{CEABCAD5-D00D-4114-8985-B83270679455}"/>
+    <hyperlink ref="F67" r:id="rId130" xr:uid="{E7946A30-8A55-4A37-B155-B6EFB266D883}"/>
+    <hyperlink ref="F112" r:id="rId131" xr:uid="{868A966A-8C31-47FD-A98D-4C402066AFB7}"/>
+    <hyperlink ref="F85" r:id="rId132" xr:uid="{6AEF366C-9DF8-4824-89B0-4C71020C0079}"/>
+    <hyperlink ref="F102" r:id="rId133" xr:uid="{B8ACDDF3-8E66-4E78-A519-C81C929AFB2F}"/>
+    <hyperlink ref="E38" r:id="rId134" display="https://www.linkedin.com/in/tricia-dockree-821b453a/" xr:uid="{DA65C1A0-887B-453C-8B5E-C6B2C12E98D4}"/>
+    <hyperlink ref="E122" r:id="rId135" display="https://www.linkedin.com/in/kristin-costanzo-931498380/" xr:uid="{F57E52E8-84BA-4F35-97F6-09377464E399}"/>
+    <hyperlink ref="E119" r:id="rId136" display="https://www.linkedin.com/in/stephen-m-bernard/" xr:uid="{3AF57711-4517-4503-80B1-3A0F825046CD}"/>
+    <hyperlink ref="E133" r:id="rId137" display="https://www.linkedin.com/in/martin-you1/" xr:uid="{CBEBCE6C-B2D9-407F-959F-3DAE94EDC039}"/>
+    <hyperlink ref="E132" r:id="rId138" display="https://www.linkedin.com/in/logan-hiskes/" xr:uid="{51677E28-B812-4A8C-BF27-C04A3E661E33}"/>
+    <hyperlink ref="E134" r:id="rId139" display="https://www.linkedin.com/in/akshita-ponnuru/" xr:uid="{DE004323-C0B5-4368-A3EA-D3597FD6FE10}"/>
+    <hyperlink ref="E135" r:id="rId140" display="https://www.linkedin.com/in/haydenmkeller/" xr:uid="{FCE3CCBF-024E-4F56-8E45-C753E4F7D1A3}"/>
+    <hyperlink ref="E136" r:id="rId141" display="https://www.linkedin.com/in/lily-notes-593653265/" xr:uid="{18860300-E773-4DB5-9605-AEDE886D3A7C}"/>
+    <hyperlink ref="E137" r:id="rId142" display="https://www.linkedin.com/in/khushipatellll/" xr:uid="{A642F3BD-569A-43D6-A2FC-731B32FEB6FA}"/>
+    <hyperlink ref="E138" r:id="rId143" display="https://www.linkedin.com/in/sanya-patel-7340bb22b/" xr:uid="{872FF9CF-9B05-485D-9F61-755D1F3A58D8}"/>
+    <hyperlink ref="E129" r:id="rId144" display="https://www.linkedin.com/in/andrea-feldmann-0095136/" xr:uid="{9D37D9FE-70DB-424B-8877-11226FEF2238}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId139"/>
+    <tablePart r:id="rId145"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4829,52 +4991,52 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>443</v>
+        <v>463</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>444</v>
+        <v>464</v>
       </c>
       <c r="B2" t="s">
-        <v>445</v>
+        <v>465</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="87">
       <c r="A3" t="s">
-        <v>446</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>447</v>
+        <v>466</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>467</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="130.5">
       <c r="A4" t="s">
-        <v>448</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>449</v>
+        <v>468</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>469</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="188.45">
       <c r="A5" t="s">
-        <v>450</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>451</v>
+        <v>470</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>471</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="43.5">
       <c r="A6" t="s">
-        <v>452</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>453</v>
+        <v>472</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>473</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>454</v>
+        <v>474</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="14.1" customHeight="1"/>
@@ -4882,39 +5044,39 @@
     <row r="10" spans="1:2" ht="14.1" customHeight="1"/>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>455</v>
+        <v>475</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>444</v>
+        <v>464</v>
       </c>
       <c r="B14" t="s">
-        <v>456</v>
+        <v>476</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="72.599999999999994">
       <c r="A15" t="s">
-        <v>457</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>458</v>
+        <v>477</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="144.94999999999999">
       <c r="A16" t="s">
-        <v>459</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>460</v>
+        <v>479</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>480</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="87">
       <c r="A17" t="s">
-        <v>461</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>462</v>
+        <v>481</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>482</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Liam Ford to employee roster
</commit_message>
<xml_diff>
--- a/assets/Strategy & Operations Service Lines.xlsx
+++ b/assets/Strategy & Operations Service Lines.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://impactadvisors3-my.sharepoint.com/personal/john_decicco_impact-advisors_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E6671365-14F0-44A3-AAEC-95154F5C909C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{19597BD0-46FE-4A48-AE67-03F5E552C09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{AAB7EEAF-11CB-4475-B2F2-A15F99F765BD}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="847" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="486">
   <si>
     <t>Name</t>
   </si>
@@ -1430,6 +1430,15 @@
   </si>
   <si>
     <t>sanya.patel@impact-advisors.com</t>
+  </si>
+  <si>
+    <t>Liam Ford</t>
+  </si>
+  <si>
+    <t>Liam Ford | LinkedIn</t>
+  </si>
+  <si>
+    <t>liam.ford@impact-advisors.com</t>
   </si>
   <si>
     <r>
@@ -1654,8 +1663,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}" name="Table1" displayName="Table1" ref="A1:F138" totalsRowShown="0">
-  <autoFilter ref="A1:F138" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}" name="Table1" displayName="Table1" ref="A1:F139" totalsRowShown="0">
+  <autoFilter ref="A1:F139" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{B7225A69-4070-43CE-AFA1-930CE8ABA093}" name="Name"/>
     <tableColumn id="2" xr3:uid="{74BF9A37-C28E-424C-A808-B2BBA42CFA48}" name="Service Line"/>
@@ -2034,7 +2043,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09DBBB96-A9E5-4CC1-B781-70890184EE77}">
-  <dimension ref="A1:I138"/>
+  <dimension ref="A1:I139"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -4815,6 +4824,26 @@
       </c>
       <c r="F138" t="s">
         <v>462</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6">
+      <c r="A139" t="s">
+        <v>463</v>
+      </c>
+      <c r="B139" t="s">
+        <v>346</v>
+      </c>
+      <c r="C139" t="s">
+        <v>442</v>
+      </c>
+      <c r="D139" t="s">
+        <v>9</v>
+      </c>
+      <c r="E139" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="F139" t="s">
+        <v>465</v>
       </c>
     </row>
   </sheetData>
@@ -4963,10 +4992,11 @@
     <hyperlink ref="E137" r:id="rId142" display="https://www.linkedin.com/in/khushipatellll/" xr:uid="{A642F3BD-569A-43D6-A2FC-731B32FEB6FA}"/>
     <hyperlink ref="E138" r:id="rId143" display="https://www.linkedin.com/in/sanya-patel-7340bb22b/" xr:uid="{872FF9CF-9B05-485D-9F61-755D1F3A58D8}"/>
     <hyperlink ref="E129" r:id="rId144" display="https://www.linkedin.com/in/andrea-feldmann-0095136/" xr:uid="{9D37D9FE-70DB-424B-8877-11226FEF2238}"/>
+    <hyperlink ref="E139" r:id="rId145" display="https://www.linkedin.com/in/liam-ford-6075b1213/" xr:uid="{574041DF-6D1D-410E-A2C3-623293E84DF3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId145"/>
+    <tablePart r:id="rId146"/>
   </tableParts>
 </worksheet>
 </file>
@@ -4991,52 +5021,52 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B2" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="87">
       <c r="A3" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="130.5">
       <c r="A4" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="188.45">
       <c r="A5" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="43.5">
       <c r="A6" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="14.1" customHeight="1"/>
@@ -5044,39 +5074,39 @@
     <row r="10" spans="1:2" ht="14.1" customHeight="1"/>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B14" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="72.599999999999994">
       <c r="A15" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="144.94999999999999">
       <c r="A16" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="87">
       <c r="A17" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update service line roster and Oracle Health label
</commit_message>
<xml_diff>
--- a/assets/Strategy & Operations Service Lines.xlsx
+++ b/assets/Strategy & Operations Service Lines.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://impactadvisors3-my.sharepoint.com/personal/john_decicco_impact-advisors_com/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://impactadvisors3.sharepoint.com/sites/2026ConsultantGoals/Shared Documents/General/Networking Toolkit/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{19597BD0-46FE-4A48-AE67-03F5E552C09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{68C97299-4DFA-478B-BCFE-4D65F399F4A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{AAB7EEAF-11CB-4475-B2F2-A15F99F765BD}"/>
   </bookViews>
@@ -1432,7 +1432,7 @@
     <t>sanya.patel@impact-advisors.com</t>
   </si>
   <si>
-    <t>Liam Ford</t>
+    <t xml:space="preserve">Liam Ford </t>
   </si>
   <si>
     <t>Liam Ford | LinkedIn</t>
@@ -4831,7 +4831,7 @@
         <v>463</v>
       </c>
       <c r="B139" t="s">
-        <v>346</v>
+        <v>85</v>
       </c>
       <c r="C139" t="s">
         <v>442</v>
@@ -4992,7 +4992,7 @@
     <hyperlink ref="E137" r:id="rId142" display="https://www.linkedin.com/in/khushipatellll/" xr:uid="{A642F3BD-569A-43D6-A2FC-731B32FEB6FA}"/>
     <hyperlink ref="E138" r:id="rId143" display="https://www.linkedin.com/in/sanya-patel-7340bb22b/" xr:uid="{872FF9CF-9B05-485D-9F61-755D1F3A58D8}"/>
     <hyperlink ref="E129" r:id="rId144" display="https://www.linkedin.com/in/andrea-feldmann-0095136/" xr:uid="{9D37D9FE-70DB-424B-8877-11226FEF2238}"/>
-    <hyperlink ref="E139" r:id="rId145" display="https://www.linkedin.com/in/liam-ford-6075b1213/" xr:uid="{574041DF-6D1D-410E-A2C3-623293E84DF3}"/>
+    <hyperlink ref="E139" r:id="rId145" display="https://www.linkedin.com/in/liam-ford-6075b1213/" xr:uid="{15B31879-B400-48DE-A3F9-1BF55BC45271}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -5116,4 +5116,193 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010062AC75732FCC574AA39F1F73CAC12435" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="63221f8ce7b9bdba850c731f1f8526dd">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="18c801aa-b08e-4147-8d71-4a4146fc5f82" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a6e5fe67e0597052bb7d02be10438d84" ns2:_="">
+    <xsd:import namespace="18c801aa-b08e-4147-8d71-4a4146fc5f82"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="18c801aa-b08e-4147-8d71-4a4146fc5f82" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="14" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{898626DD-6B53-4F3D-BC27-4B5A8D32B3B3}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFA9E554-1ADE-46CE-8803-AC258E13C25F}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{887352FC-8020-462A-8C14-3CDA6EDFB226}"/>
 </file>
</xml_diff>

<commit_message>
Update roster with Holly Ezell
</commit_message>
<xml_diff>
--- a/assets/Strategy & Operations Service Lines.xlsx
+++ b/assets/Strategy & Operations Service Lines.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://impactadvisors3.sharepoint.com/sites/2026ConsultantGoals/Shared Documents/General/Networking Toolkit/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://impactadvisors3-my.sharepoint.com/personal/martin_you_impact-advisors_com/Documents/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{68C97299-4DFA-478B-BCFE-4D65F399F4A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A49A3C7-4F9F-4959-85D2-6CD16742BA05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{AAB7EEAF-11CB-4475-B2F2-A15F99F765BD}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="859" uniqueCount="490">
   <si>
     <t>Name</t>
   </si>
@@ -1563,12 +1563,24 @@
 • Enforce workflows &amp; improve operations: ensure SOP adherence and drive targeted process improvement
 • Partner with client delivery on engagement success</t>
   </si>
+  <si>
+    <t>Holly Ezell</t>
+  </si>
+  <si>
+    <t>Nashville</t>
+  </si>
+  <si>
+    <t>Holly Ezell | LinkedIn</t>
+  </si>
+  <si>
+    <t>Holly.ezell@impact-advisors.com</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1663,8 +1675,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}" name="Table1" displayName="Table1" ref="A1:F139" totalsRowShown="0">
-  <autoFilter ref="A1:F139" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}" name="Table1" displayName="Table1" ref="A1:F140" totalsRowShown="0">
+  <autoFilter ref="A1:F140" xr:uid="{8700CBAD-FC9E-4C75-BB7D-18040C7D2A47}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{B7225A69-4070-43CE-AFA1-930CE8ABA093}" name="Name"/>
     <tableColumn id="2" xr3:uid="{74BF9A37-C28E-424C-A808-B2BBA42CFA48}" name="Service Line"/>
@@ -2043,19 +2055,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09DBBB96-A9E5-4CC1-B781-70890184EE77}">
-  <dimension ref="A1:I139"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:I140"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="55.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="40.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="48.85546875" customWidth="1"/>
+    <col min="1" max="1" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="55.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="40.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="48.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2075,7 +2087,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2098,7 +2110,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -2121,7 +2133,7 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -2144,7 +2156,7 @@
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -2167,7 +2179,7 @@
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>26</v>
       </c>
@@ -2190,7 +2202,7 @@
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -2210,7 +2222,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>34</v>
       </c>
@@ -2230,7 +2242,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>37</v>
       </c>
@@ -2250,7 +2262,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>41</v>
       </c>
@@ -2270,7 +2282,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -2290,7 +2302,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>48</v>
       </c>
@@ -2310,7 +2322,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>52</v>
       </c>
@@ -2330,7 +2342,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>56</v>
       </c>
@@ -2350,7 +2362,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>60</v>
       </c>
@@ -2370,7 +2382,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>63</v>
       </c>
@@ -2390,7 +2402,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>67</v>
       </c>
@@ -2410,7 +2422,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>70</v>
       </c>
@@ -2430,7 +2442,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>74</v>
       </c>
@@ -2450,7 +2462,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>78</v>
       </c>
@@ -2470,7 +2482,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>81</v>
       </c>
@@ -2490,7 +2502,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>84</v>
       </c>
@@ -2510,7 +2522,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>89</v>
       </c>
@@ -2530,7 +2542,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>93</v>
       </c>
@@ -2550,7 +2562,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>96</v>
       </c>
@@ -2570,7 +2582,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>99</v>
       </c>
@@ -2590,7 +2602,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>102</v>
       </c>
@@ -2610,7 +2622,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>105</v>
       </c>
@@ -2630,7 +2642,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>109</v>
       </c>
@@ -2650,7 +2662,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>113</v>
       </c>
@@ -2670,7 +2682,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>116</v>
       </c>
@@ -2690,7 +2702,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>120</v>
       </c>
@@ -2710,7 +2722,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>124</v>
       </c>
@@ -2730,7 +2742,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>128</v>
       </c>
@@ -2750,7 +2762,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>132</v>
       </c>
@@ -2768,7 +2780,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>135</v>
       </c>
@@ -2788,7 +2800,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>138</v>
       </c>
@@ -2808,7 +2820,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>141</v>
       </c>
@@ -2828,7 +2840,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>145</v>
       </c>
@@ -2848,7 +2860,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>149</v>
       </c>
@@ -2868,7 +2880,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>153</v>
       </c>
@@ -2888,7 +2900,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>156</v>
       </c>
@@ -2908,7 +2920,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>159</v>
       </c>
@@ -2928,7 +2940,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>162</v>
       </c>
@@ -2948,7 +2960,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>166</v>
       </c>
@@ -2968,7 +2980,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>170</v>
       </c>
@@ -2988,7 +3000,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>174</v>
       </c>
@@ -3008,7 +3020,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>177</v>
       </c>
@@ -3028,7 +3040,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>180</v>
       </c>
@@ -3048,7 +3060,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>184</v>
       </c>
@@ -3068,7 +3080,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>187</v>
       </c>
@@ -3088,7 +3100,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>190</v>
       </c>
@@ -3108,7 +3120,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>194</v>
       </c>
@@ -3128,7 +3140,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>197</v>
       </c>
@@ -3148,7 +3160,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>200</v>
       </c>
@@ -3168,7 +3180,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>203</v>
       </c>
@@ -3188,7 +3200,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>206</v>
       </c>
@@ -3208,7 +3220,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>210</v>
       </c>
@@ -3228,7 +3240,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>213</v>
       </c>
@@ -3248,7 +3260,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>81</v>
       </c>
@@ -3268,7 +3280,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>216</v>
       </c>
@@ -3288,7 +3300,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>220</v>
       </c>
@@ -3308,7 +3320,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>223</v>
       </c>
@@ -3328,7 +3340,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>226</v>
       </c>
@@ -3348,7 +3360,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>230</v>
       </c>
@@ -3368,7 +3380,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>233</v>
       </c>
@@ -3388,7 +3400,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>236</v>
       </c>
@@ -3408,7 +3420,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>239</v>
       </c>
@@ -3428,7 +3440,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>242</v>
       </c>
@@ -3448,7 +3460,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>246</v>
       </c>
@@ -3468,7 +3480,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>250</v>
       </c>
@@ -3488,7 +3500,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>253</v>
       </c>
@@ -3508,7 +3520,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>60</v>
       </c>
@@ -3528,7 +3540,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>256</v>
       </c>
@@ -3548,7 +3560,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>259</v>
       </c>
@@ -3568,7 +3580,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>262</v>
       </c>
@@ -3588,7 +3600,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>265</v>
       </c>
@@ -3608,7 +3620,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>78</v>
       </c>
@@ -3628,7 +3640,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>268</v>
       </c>
@@ -3648,7 +3660,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>271</v>
       </c>
@@ -3668,7 +3680,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="81" spans="1:6">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>276</v>
       </c>
@@ -3688,7 +3700,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="82" spans="1:6">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>279</v>
       </c>
@@ -3708,7 +3720,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="83" spans="1:6">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>282</v>
       </c>
@@ -3728,7 +3740,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="84" spans="1:6">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>285</v>
       </c>
@@ -3748,7 +3760,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>288</v>
       </c>
@@ -3768,7 +3780,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="86" spans="1:6">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>291</v>
       </c>
@@ -3788,7 +3800,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="87" spans="1:6">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>294</v>
       </c>
@@ -3808,7 +3820,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="88" spans="1:6">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>297</v>
       </c>
@@ -3828,7 +3840,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="89" spans="1:6">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>300</v>
       </c>
@@ -3848,7 +3860,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="90" spans="1:6">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>303</v>
       </c>
@@ -3868,7 +3880,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="91" spans="1:6">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>307</v>
       </c>
@@ -3888,7 +3900,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>311</v>
       </c>
@@ -3906,7 +3918,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="93" spans="1:6">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>313</v>
       </c>
@@ -3926,7 +3938,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>316</v>
       </c>
@@ -3946,7 +3958,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="95" spans="1:6">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>319</v>
       </c>
@@ -3966,7 +3978,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="96" spans="1:6">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>323</v>
       </c>
@@ -3986,7 +3998,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="97" spans="1:6">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>326</v>
       </c>
@@ -4006,7 +4018,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="98" spans="1:6">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>330</v>
       </c>
@@ -4026,7 +4038,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="99" spans="1:6">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>333</v>
       </c>
@@ -4046,7 +4058,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="100" spans="1:6">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>336</v>
       </c>
@@ -4066,7 +4078,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="101" spans="1:6">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>339</v>
       </c>
@@ -4086,7 +4098,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="102" spans="1:6">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>342</v>
       </c>
@@ -4106,7 +4118,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="103" spans="1:6">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>345</v>
       </c>
@@ -4126,7 +4138,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="104" spans="1:6">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>349</v>
       </c>
@@ -4146,7 +4158,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="105" spans="1:6">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>352</v>
       </c>
@@ -4166,7 +4178,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="106" spans="1:6">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
         <v>355</v>
       </c>
@@ -4186,7 +4198,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="107" spans="1:6">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>358</v>
       </c>
@@ -4206,7 +4218,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="108" spans="1:6">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>361</v>
       </c>
@@ -4226,7 +4238,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="109" spans="1:6">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>364</v>
       </c>
@@ -4246,7 +4258,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="110" spans="1:6">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>367</v>
       </c>
@@ -4266,7 +4278,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="111" spans="1:6">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>370</v>
       </c>
@@ -4286,7 +4298,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="112" spans="1:6">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
         <v>373</v>
       </c>
@@ -4306,7 +4318,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="113" spans="1:6">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>376</v>
       </c>
@@ -4326,7 +4338,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="114" spans="1:6">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
         <v>380</v>
       </c>
@@ -4346,7 +4358,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="115" spans="1:6">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>383</v>
       </c>
@@ -4366,7 +4378,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="116" spans="1:6">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>386</v>
       </c>
@@ -4386,7 +4398,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="117" spans="1:6">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>391</v>
       </c>
@@ -4406,7 +4418,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="118" spans="1:6">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>394</v>
       </c>
@@ -4426,7 +4438,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="119" spans="1:6">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>398</v>
       </c>
@@ -4446,7 +4458,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="120" spans="1:6">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>402</v>
       </c>
@@ -4466,7 +4478,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="121" spans="1:6">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>407</v>
       </c>
@@ -4486,7 +4498,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="122" spans="1:6">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>410</v>
       </c>
@@ -4506,7 +4518,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="123" spans="1:6">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>413</v>
       </c>
@@ -4526,7 +4538,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="124" spans="1:6">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>416</v>
       </c>
@@ -4546,7 +4558,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="125" spans="1:6">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>419</v>
       </c>
@@ -4566,7 +4578,7 @@
         <v>421</v>
       </c>
     </row>
-    <row r="126" spans="1:6">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>422</v>
       </c>
@@ -4586,7 +4598,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="127" spans="1:6">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>425</v>
       </c>
@@ -4606,7 +4618,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="128" spans="1:6">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>428</v>
       </c>
@@ -4626,7 +4638,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="129" spans="1:6">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>431</v>
       </c>
@@ -4646,7 +4658,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="130" spans="1:6">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>435</v>
       </c>
@@ -4666,7 +4678,7 @@
         <v>437</v>
       </c>
     </row>
-    <row r="131" spans="1:6">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>438</v>
       </c>
@@ -4686,7 +4698,7 @@
         <v>440</v>
       </c>
     </row>
-    <row r="132" spans="1:6">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>441</v>
       </c>
@@ -4706,7 +4718,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="133" spans="1:6">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>445</v>
       </c>
@@ -4726,7 +4738,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="134" spans="1:6">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>448</v>
       </c>
@@ -4746,7 +4758,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="135" spans="1:6">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>451</v>
       </c>
@@ -4766,7 +4778,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="136" spans="1:6">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>454</v>
       </c>
@@ -4786,7 +4798,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="137" spans="1:6">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>457</v>
       </c>
@@ -4806,7 +4818,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="138" spans="1:6">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>460</v>
       </c>
@@ -4826,7 +4838,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="139" spans="1:6">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>463</v>
       </c>
@@ -4844,6 +4856,26 @@
       </c>
       <c r="F139" t="s">
         <v>465</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A140" t="s">
+        <v>486</v>
+      </c>
+      <c r="B140" t="s">
+        <v>346</v>
+      </c>
+      <c r="C140" t="s">
+        <v>13</v>
+      </c>
+      <c r="D140" t="s">
+        <v>487</v>
+      </c>
+      <c r="E140" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="F140" s="1" t="s">
+        <v>489</v>
       </c>
     </row>
   </sheetData>
@@ -4993,10 +5025,12 @@
     <hyperlink ref="E138" r:id="rId143" display="https://www.linkedin.com/in/sanya-patel-7340bb22b/" xr:uid="{872FF9CF-9B05-485D-9F61-755D1F3A58D8}"/>
     <hyperlink ref="E129" r:id="rId144" display="https://www.linkedin.com/in/andrea-feldmann-0095136/" xr:uid="{9D37D9FE-70DB-424B-8877-11226FEF2238}"/>
     <hyperlink ref="E139" r:id="rId145" display="https://www.linkedin.com/in/liam-ford-6075b1213/" xr:uid="{15B31879-B400-48DE-A3F9-1BF55BC45271}"/>
+    <hyperlink ref="E140" r:id="rId146" xr:uid="{EA224624-EE80-4FC0-8A49-F7F1CA6414B2}"/>
+    <hyperlink ref="F140" r:id="rId147" xr:uid="{0692CBCB-6A78-42AD-A3D0-B5B9DE759520}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId146"/>
+    <tablePart r:id="rId148"/>
   </tableParts>
 </worksheet>
 </file>
@@ -5004,7 +5038,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{872BEBDA-C4A6-41BA-99D6-EF41FC49D676}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5013,18 +5047,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17E0BE01-2F8D-414B-AC76-04271BD349CD}">
   <dimension ref="A1:B17"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="46.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="87.85546875" customWidth="1"/>
+    <col min="1" max="1" width="46.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="87.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>467</v>
       </c>
@@ -5032,7 +5066,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="87">
+    <row r="3" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>469</v>
       </c>
@@ -5040,7 +5074,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="130.5">
+    <row r="4" spans="1:2" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>471</v>
       </c>
@@ -5048,7 +5082,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="188.45">
+    <row r="5" spans="1:2" ht="188.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>473</v>
       </c>
@@ -5056,7 +5090,7 @@
         <v>474</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="43.5">
+    <row r="6" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>475</v>
       </c>
@@ -5064,20 +5098,20 @@
         <v>476</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>477</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="14.1" customHeight="1"/>
-    <row r="9" spans="1:2" ht="14.1" customHeight="1"/>
-    <row r="10" spans="1:2" ht="14.1" customHeight="1"/>
-    <row r="13" spans="1:2">
+    <row r="8" spans="1:2" ht="14.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="1:2" ht="14.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="10" spans="1:2" ht="14.15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>478</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>467</v>
       </c>
@@ -5085,7 +5119,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="72.599999999999994">
+    <row r="15" spans="1:2" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>480</v>
       </c>
@@ -5093,7 +5127,7 @@
         <v>481</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="144.94999999999999">
+    <row r="16" spans="1:2" ht="145" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>482</v>
       </c>
@@ -5101,7 +5135,7 @@
         <v>483</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="87">
+    <row r="17" spans="1:2" ht="87" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>484</v>
       </c>
@@ -5119,21 +5153,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010062AC75732FCC574AA39F1F73CAC12435" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="63221f8ce7b9bdba850c731f1f8526dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="18c801aa-b08e-4147-8d71-4a4146fc5f82" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a6e5fe67e0597052bb7d02be10438d84" ns2:_="">
     <xsd:import namespace="18c801aa-b08e-4147-8d71-4a4146fc5f82"/>
@@ -5295,14 +5314,59 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{898626DD-6B53-4F3D-BC27-4B5A8D32B3B3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{887352FC-8020-462A-8C14-3CDA6EDFB226}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="18c801aa-b08e-4147-8d71-4a4146fc5f82"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFA9E554-1ADE-46CE-8803-AC258E13C25F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFA9E554-1ADE-46CE-8803-AC258E13C25F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="18c801aa-b08e-4147-8d71-4a4146fc5f82"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{887352FC-8020-462A-8C14-3CDA6EDFB226}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{898626DD-6B53-4F3D-BC27-4B5A8D32B3B3}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>